<commit_message>
feat(P6): Pelvis 회전 3종 표준화 + Feature_Dictionary Category 단일화
- Feature_Dictionary: Group/Object 분리 → Category 단일 컬럼 (Body 폐기)
  규모 확대 시 Body/Upper Limb/Club 계층으로 확장 (Naming_Rule에 명시)
- P6 표준화 추가(6섹션): Pelvis Rotation Insufficient / Excessive / Stall
  → 총 6/28 완료 (Pelvis Open Early·Rotation Insuf/Excess·Stall·Early Extension·High Hands)
- 신규 Mechanism 없이 기존 Dictionary 재사용(M-PRS/ROT/ARM/CLB/CMP 계열)
  → Dictionary 안정화 신호. Pelvis Stall↔Handle Stall 양방향 Co-occurrence 명시
- P6 블록 순서/타이틀에서 Body 그룹 표기 제거 (Object/Attribute만)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/DOH_Knowledge.xlsx
+++ b/DOH_Knowledge.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TODO'!$A$1:$E$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B115"/>
+  <dimension ref="A1:B149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -604,7 +604,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Pelvis Open Early  (골반 조기 오픈)   ·   Body / Pelvis / Rotation/Timing · Early</t>
+          <t>Pelvis Open Early  (골반 조기 오픈)   ·   Pelvis / Rotation/Timing · Early</t>
         </is>
       </c>
     </row>
@@ -792,194 +792,245 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Pelvis Rotation Insufficient  (골반 회전 부족)   ·   Body / Pelvis / Rotation/Amount · Insufficient</t>
+          <t>Pelvis Rotation Insufficient  (골반 회전 부족)   ·   Pelvis / Rotation/Amount · Insufficient</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 정의</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Pelvis Rotation Excessive  (골반 과회전)   ·   Body / Pelvis / Rotation/Amount · Excessive</t>
+          <t>다운스윙 중반(P6)에서 골반의 회전량이 정상보다 부족한 현상. 회전 시점(Timing)이나 속도(Velocity)가 아니라 회전량(Amount)이 핵심이다. 흉곽 회전 부족과는 독립 Feature로 유지한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Pelvis Rotation Insufficient (골반 회전 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Late Pressure Shift (압력 이동 지연)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+Pelvis Rotation Insufficient (골반 회전 부족)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A19" s="4" t="inlineStr"/>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Pelvis Stall  (골반 회전 정지)   ·   Body / Pelvis / Rotation/Velocity · Stall</t>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+Pressure Remains On The Trail Side.
+(압력이 트레일측에 남아있다.)
+   ↓
+Pelvis Rotation Insufficient (골반 회전 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+Thorax Rotation Does Not Complete Through Impact.
+(흉곽 회전이 임팩트까지 완성되지 않는다.)
+   ↓
+Pelvis Rotation Insufficient (골반 회전 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Pelvis Rotation Insufficient (골반 회전 부족)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Spin-out  (스핀아웃)   ·   Body / Pelvis / Pattern · Spin-out</t>
+          <t>Pelvis Rotation Insufficient (골반 회전 부족)
+   ↓
+Arm Delivery Space Is Reduced.
+(팔이 내려올 공간이 감소한다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Insufficient (골반 회전 부족)
+   ↓
+The Hands Take Over Club Delivery.
+(손이 클럽 전달을 주도한다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Insufficient (골반 회전 부족)
+   ↓
+The Arms Compensate For Delayed Body Motion.
+(몸의 지연을 팔이 보상한다.)
+   ↓
+Casting (캐스팅)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A25" s="4" t="inlineStr"/>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Early Extension  (얼리 익스텐션)   ·   Body / Pelvis / Pattern · Early Extension</t>
+          <t>Pelvis Rotation Insufficient (골반 회전 부족)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈) / Club Face Closed (클럽페이스 클로즈)  ※보상 방식에 따라</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>· Thorax Rotation Insufficient (흉곽 회전 부족) — 강한 동반, 단 독립 축으로 유지
+· Hanging Back (체중 뒤잔류)
+· Late Release (늦은 릴리즈)
+· Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Rotation Insufficient와 Thorax Rotation Insufficient 중 어느 쪽이 선행 원인인 경우가 많은지 검증 필요.
+· 회전 부족 골퍼의 Subtype: Slide 보상형 vs 팔 사용(Casting) 보상형 분리 가능성.
+· 리드측 압력은 충분하지만 회전만 부족한 유형(Hanging Back 비동반) 존재 여부 확인.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>· 골반 3축(Amount/Timing/Velocity) 중 Amount 축. Pelvis와 Thorax의 Rotation Insufficient는 강한 Co-occurrence이나 독립 Feature로 유지한다.
+· 회전 부족 → 팔·손 보상(M-CMP 계열) 경로가 반복되므로 보상 언어를 표준으로 재사용한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Excessive  (골반 과회전)   ·   Pelvis / Rotation/Amount · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>■ 정의</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 골반이 볼 방향으로 전진하거나 고관절 굴곡이 조기에 소실되며 몸이 일찍 일어나는 현상. 골반·고관절·척추 자세를 유지하지 못하고 신체가 조기에 신전되는 것이 핵심이다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반의 회전량이 정상보다 과도한 현상. 회전량만 많은 상태이며, 체중이동·시퀀스·클럽 전달까지 무너진 복합 현상인 Spin-out과는 구분한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>■ 원인 추정</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Lead Pressure Insufficient (리드측 압력 부족)
-   ↓
-Pressure Does Not Reach The Lead Side Before Impact.
-(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
-   ↓
-Early Extension (얼리 익스텐션)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr"/>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Pelvis Stall (골반 회전 정지)
-   ↓
-Pelvis Rotation Decelerates Before Impact.
-(임팩트 전에 골반 회전이 감속한다.)
-   ↓
-The Lead Side Cannot Become The Primary Rotation Axis.
-(리드측이 주 회전축이 되지 못한다.)
-   ↓
-Early Extension (얼리 익스텐션)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Arm Stuck (팔 끼임)
-   ↓
-The Body Loses Delivery Space.
-(다운스윙 공간이 부족해진다.)
-   ↓
-The Body Extends Early To Create Space.
-(공간을 만들기 위해 몸이 일찍 신전한다.)
-   ↓
-Early Extension (얼리 익스텐션)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr"/>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Steep Shaft (가파른 샤프트)
-   ↓
-The Body Extends Early To Create Space.
-(공간을 만들기 위해 몸이 일찍 신전한다.)
-   ↓
-Early Extension (얼리 익스텐션)</t>
+          <t>Lead Pressure Excessive (리드측 압력 과다)
+   ↓
+Pressure On The Lead Side Becomes Excessive.
+(리드측 압력이 과도해진다.)
+   ↓
+Pelvis Rotation Excessive (골반 과회전)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>■ 이후 나타날 가능성</t>
-        </is>
-      </c>
+      <c r="A33" s="4" t="inlineStr"/>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Early Extension (얼리 익스텐션)
-   ↓
-The Body Loses Delivery Space.
-(다운스윙 공간이 부족해진다.)
-   ↓
-Handle Raise (핸들 상승)</t>
+          <t>Trail Leg Push Excessive (트레일 다리 추진 과다)
+   ↓
+Trail Leg Drive Opens The Pelvis Early.
+(트레일 다리의 추진이 골반을 조기에 연다.)
+   ↓
+Pelvis Rotation Excessive (골반 과회전)</t>
         </is>
       </c>
     </row>
@@ -987,14 +1038,12 @@
       <c r="A34" s="4" t="inlineStr"/>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Early Extension (얼리 익스텐션)
-   ↓
-The Arms Fall Behind The Rotating Body.
-(회전하는 몸에 비해 팔이 뒤처진다.)
-   ↓
-Arm Stuck (팔 끼임)
-   ↓
-Late Release (늦은 릴리즈)</t>
+          <t>Thorax Rotation Excessive (흉곽 과회전)
+   ↓
+Body Rotation Leads The Downswing.
+(몸통 회전이 다운스윙을 주도한다.)
+   ↓
+Pelvis Rotation Excessive (골반 과회전)</t>
         </is>
       </c>
     </row>
@@ -1002,20 +1051,468 @@
       <c r="A35" s="4" t="inlineStr"/>
       <c r="B35" s="4" t="inlineStr">
         <is>
+          <t>Body Rotation Dominant (몸통 회전 주도)
+   ↓
+Body Rotation Leads The Downswing.
+(몸통 회전이 다운스윙을 주도한다.)
+   ↓
+Pelvis Rotation Excessive (골반 과회전)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Excessive (골반 과회전)
+   ↓
+The Pelvis Rotates Faster Than The Arms Can Follow.
+(팔이 따라올 수 없을 만큼 골반이 빠르게 회전한다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Handle Raise (핸들 상승)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr"/>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Excessive (골반 과회전)
+   ↓
+Thorax Rotation Outpaces Arm Delivery.
+(흉곽 회전이 팔 전달보다 앞선다.)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Excessive (골반 과회전)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr"/>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Excessive (골반 과회전)
+   ↓
+The Body Rotates Around The Trail Side.
+(몸이 트레일측을 중심으로 회전한다.)
+   ↓
+Spin-out (스핀아웃)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Open Early (골반 조기 오픈) — 회전량과 타이밍 동반형
+· Thorax Rotation Excessive (흉곽 과회전)
+· Spin-out (스핀아웃)
+· Club Face Open (클럽페이스 오픈)
+· Handle Raise (핸들 상승)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Rotation Excessive와 Pelvis Open Early는 자주 함께 나타나지만, 회전량은 많아도 타이밍은 정상인 골퍼가 존재.
+· 과회전이 항상 Club Face Open을 유발하지는 않음 — 손·팔 릴리즈가 좋은 골퍼는 보상 가능.
+· Trail Leg Push Excessive를 독립 Feature로 둘지 검토 (현재는 원인 후보로 유지).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>· 회전량만 많은 것(Excessive)과 회전량+시퀀스 붕괴(Spin-out)를 반드시 구분한다.
+· Trail Leg Drive(트레일 다리의 추진이 골반을 조기에 연다)는 Pelvis Open Early와 Pelvis Rotation Excessive의 공통 원인으로 재사용되는 표준 Mechanism이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Pelvis Stall  (골반 회전 정지)   ·   Pelvis / Rotation/Velocity · Stall</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반 회전이 정상보다 일찍 감속하거나 정지하는 현상. 회전량(Amount)이 아니라 회전 속도(Velocity)가 유지되지 못하는 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Pelvis Stall (골반 회전 정지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
           <t>Early Extension (얼리 익스텐션)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Pelvis Stall (골반 회전 정지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+Pressure Remains On The Trail Side.
+(압력이 트레일측에 남아있다.)
+   ↓
+Pelvis Stall (골반 회전 정지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Stall (흉곽 회전 정지)
+   ↓
+Thorax Rotation Decelerates Before Impact.
+(임팩트 전에 흉곽 회전이 감속한다.)
+   ↓
+Pelvis Stall (골반 회전 정지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+Pelvis Rotation Decelerates Before Impact.
+(임팩트 전에 골반 회전이 감속한다.)
+   ↓
+Handle Stall (핸들 정지)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr"/>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr"/>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+The Hands Take Over Club Delivery.
+(손이 클럽 전달을 주도한다.)
+   ↓
+Casting (캐스팅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr"/>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Stall (골반 회전 정지)
    ↓
 The Body Extends Early To Create Space.
 (공간을 만들기 위해 몸이 일찍 신전한다.)
    ↓
+Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>· Handle Stall (핸들 정지) — 선후 개인차, 양방향 연관(Bidirectional Co-occurrence)
+· Thorax Stall (흉곽 회전 정지)
+· Early Extension (얼리 익스텐션)
+· Flip Release (플립 릴리즈)
+· Hanging Back (체중 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Stall 이후 항상 Handle Stall이 오는지, 일부는 팔 속도(Casting/Arm Throw)로 보상하는지 검증.
+· Pelvis Stall과 Early Extension의 선행 관계는 개인차.
+· 완전 정지 유형 vs 단순 감속 유형 세분 필요성 검토.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>· 골반 3축 중 Velocity 축. Pelvis Stall과 Handle Stall은 선후관계가 골퍼마다 달라 일방향 인과보다 Graph에서 양방향 연관으로 관리하는 것이 현실적.
+· Pelvis Stall과 Thorax Stall은 강한 Co-occurrence이나 독립 Feature로 유지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Spin-out  (스핀아웃)   ·   Pelvis / Pattern · Spin-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Early Extension  (얼리 익스텐션)   ·   Pelvis / Pattern · Early Extension</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반이 볼 방향으로 전진하거나 고관절 굴곡이 조기에 소실되며 몸이 일찍 일어나는 현상. 골반·고관절·척추 자세를 유지하지 못하고 신체가 조기에 신전되는 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr"/>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+Pelvis Rotation Decelerates Before Impact.
+(임팩트 전에 골반 회전이 감속한다.)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr"/>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Arm Stuck (팔 끼임)
+   ↓
+The Body Loses Delivery Space.
+(다운스윙 공간이 부족해진다.)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
+Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr"/>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
+Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Body Loses Delivery Space.
+(다운스윙 공간이 부족해진다.)
+   ↓
+Handle Raise (핸들 상승)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr"/>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr"/>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
 Spine Extension Excessive (척추 과신전)
    ↓
 Head Elevation (머리 상승)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr"/>
-      <c r="B36" s="4" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr"/>
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>Early Extension (얼리 익스텐션)
    ↓
@@ -1026,13 +1523,13 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>■ Strong Co-occurrence</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>· Pelvis Stall (골반 회전 정지) — 선후 개인차, 매우 높은 동반
 · Spine Extension Excessive (척추 과신전) — 분절만 다른 동반 신전
@@ -1041,13 +1538,13 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>■ 추가 검증 포인트</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>· Early Extension은 원인이 여러 갈래(Pelvis/Space/Balance/Shaft)이므로 '왜 일어났는가'를 함께 기록해야 Graph 품질이 오른다.
 · Pelvis Stall과 Early Extension의 선행 관계는 개인차 → Strong Co-occurrence로 관리.
@@ -1055,314 +1552,314 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>■ 사고확장</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>· Early Extension은 In-degree·Out-degree가 모두 높은 Hub Node. Subtype(Pelvis / Space / Balance / Shaft Type)을 태그로 관리.
 · 공통 보상 언어 'The Body Extends Early To Create Space.'는 Spine Extension Excessive·Head Elevation 등 다수 Feature에서 재사용된다.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="1" t="inlineStr">
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Thorax Rotation Insufficient  (흉곽 회전 부족)   ·   Body / Thorax / Rotation/Amount · Insufficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Thorax Rotation Excessive  (흉곽 과회전)   ·   Body / Thorax / Rotation/Amount · Excessive</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Thorax Stall  (흉곽 회전 정지)   ·   Body / Thorax / Rotation/Velocity · Stall</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Thorax Open Early  (흉곽 조기 오픈)   ·   Body / Thorax / Rotation/Timing · Early</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Spine Extension Excessive  (척추 과신전)   ·   Body / Spine / Magnitude · Excessive</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Head Elevation  (머리 상승)   ·   Body / Head / Position/Height · Rise</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Head Drop  (머리 하강)   ·   Body / Head / Position/Height · Drop</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Head Hanging Back  (머리 뒤잔류)   ·   Body / Head / Position/Location · Trail</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="22" customHeight="1">
-      <c r="A65" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Lead Pressure Insufficient  (리드측 압력 부족)   ·   Body / Pressure / Location/Magnitude · Lead·Insufficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Lead Pressure Excessive  (리드측 압력 과다)   ·   Body / Pressure / Location/Magnitude · Lead·Excessive</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>Incomplete Pressure Transfer  (압력 이동 미완성)   ·   Body / Pressure / Timing · Late</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>High Hands  (손 높음)   ·   Upper Limb / Hands / Position/Height · High (Relative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="inlineStr">
-        <is>
-          <t>■ 정의</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 높은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 충분히 하강하지 못한 상대 위치가 핵심이다.</t>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient  (흉곽 회전 부족)   ·   Thorax / Rotation/Amount · Insufficient</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Excessive  (흉곽 과회전)   ·   Thorax / Rotation/Amount · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Thorax Stall  (흉곽 회전 정지)   ·   Thorax / Rotation/Velocity · Stall</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Thorax Open Early  (흉곽 조기 오픈)   ·   Thorax / Rotation/Timing · Early</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Spine Extension Excessive  (척추 과신전)   ·   Spine / Magnitude · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Head Elevation  (머리 상승)   ·   Head / Position/Height · Rise</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Head Drop  (머리 하강)   ·   Head / Position/Height · Drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Head Hanging Back  (머리 뒤잔류)   ·   Head / Position/Location · Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient  (리드측 압력 부족)   ·   Pressure / Location/Magnitude · Lead·Insufficient</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive  (리드측 압력 과다)   ·   Pressure / Location/Magnitude · Lead·Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Incomplete Pressure Transfer  (압력 이동 미완성)   ·   Pressure / Timing · Late</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>High Hands  (손 높음)   ·   Hands / Position/Height · High (Relative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 높은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 충분히 하강하지 못한 상대 위치가 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
           <t>■ 원인 추정</t>
         </is>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B110" s="4" t="inlineStr">
         <is>
           <t>Arm Depth Excessive (P4, 백스윙 손 과도한 깊이)
    ↓
@@ -1379,9 +1876,9 @@
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr"/>
-      <c r="B77" s="4" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr"/>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>Arm Drop Insufficient (팔 하강 부족)
    ↓
@@ -1392,9 +1889,9 @@
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr"/>
-      <c r="B78" s="4" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr"/>
+      <c r="B112" s="4" t="inlineStr">
         <is>
           <t>Early Extension (얼리 익스텐션)
    ↓
@@ -1405,13 +1902,13 @@
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="3" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -1422,9 +1919,9 @@
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr"/>
-      <c r="B80" s="4" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr"/>
+      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -1435,9 +1932,9 @@
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr"/>
-      <c r="B81" s="4" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr"/>
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -1450,9 +1947,9 @@
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="4" t="inlineStr"/>
-      <c r="B82" s="4" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr"/>
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -1463,13 +1960,13 @@
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="3" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
         <is>
           <t>■ Strong Co-occurrence</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B117" s="4" t="inlineStr">
         <is>
           <t>· Steep Shaft (가파른 샤프트)
 · Handle Raise (핸들 상승)
@@ -1478,267 +1975,267 @@
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
         <is>
           <t>■ 추가 검증 포인트</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>· High Hands가 '손이 높아서'인지 '몸의 회전에 비해 손이 늦게 내려와서'인지 레슨 데이터로 구분 필요 (후자 가능성 높음).
 · High Hands → Steep Shaft는 흔한 조합이나, 높은 손에서도 샤프트를 눕혀 전달하는 예외 골퍼 존재 여부 확인.</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="3" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
         <is>
           <t>■ 사고확장</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B119" s="4" t="inlineStr">
         <is>
           <t>· P6 손 위치 Feature는 모두 상대 위치(Relative Position): '이 시점의 다운스윙 진행에서 정상이라면 손이 어디 있어야 하는가' 기준. High/Low/Deep/Shallow 전부 동일 철학.
 · High Hands는 P4→Transition→P6를 잇는 Cross-Phase Chain의 대표 사례. P7 Steep Shaft/Outside Delivery로 이어진다.</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="22" customHeight="1">
-      <c r="A87" s="1" t="inlineStr">
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>Low Hands  (손 낮음)   ·   Upper Limb / Hands / Position/Height · Low (Relative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="3" t="inlineStr">
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Low Hands  (손 낮음)   ·   Hands / Position/Height · Low (Relative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B122" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="22" customHeight="1">
-      <c r="A90" s="1" t="inlineStr">
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>Deep Hands  (손 깊음)   ·   Upper Limb / Hands / Position/Depth · Deep</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Deep Hands  (손 깊음)   ·   Hands / Position/Depth · Deep</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B91" s="4" t="inlineStr">
+      <c r="B125" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="1" t="inlineStr">
+    <row r="127" ht="22" customHeight="1">
+      <c r="A127" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>Forward Hands  (손 전방)   ·   Upper Limb / Hands / Position/Direction · Forward</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="3" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Forward Hands  (손 전방)   ·   Hands / Position/Direction · Forward</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B128" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="22" customHeight="1">
-      <c r="A96" s="1" t="inlineStr">
+    <row r="130" ht="22" customHeight="1">
+      <c r="A130" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>Hands Too Far From Body  (손이 몸에서 멀어짐)   ·   Upper Limb / Hands / Relationship · Far</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Hands Too Far From Body  (손이 몸에서 멀어짐)   ·   Hands / Relationship · Far</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B97" s="4" t="inlineStr">
+      <c r="B131" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="22" customHeight="1">
-      <c r="A99" s="1" t="inlineStr">
+    <row r="133" ht="22" customHeight="1">
+      <c r="A133" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>Hands Too Close To Body  (손이 몸에 가까움)   ·   Upper Limb / Hands / Relationship · Close</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="3" t="inlineStr">
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body  (손이 몸에 가까움)   ·   Hands / Relationship · Close</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B134" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="1" t="inlineStr">
+    <row r="136" ht="22" customHeight="1">
+      <c r="A136" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>Late Arm  (팔 하강 지연)   ·   Upper Limb / Arm / Timing · Late</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Late Arm  (팔 하강 지연)   ·   Arm / Timing · Late</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B103" s="4" t="inlineStr">
+      <c r="B137" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="22" customHeight="1">
-      <c r="A105" s="1" t="inlineStr">
+    <row r="139" ht="22" customHeight="1">
+      <c r="A139" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>Trail Elbow Behind Body  (트레일 팔꿈치 뒤처짐)   ·   Upper Limb / Trail Elbow / Location · Trail</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="3" t="inlineStr">
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Trail Elbow Behind Body  (트레일 팔꿈치 뒤처짐)   ·   Trail Elbow / Location · Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B106" s="4" t="inlineStr">
+      <c r="B140" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="22" customHeight="1">
-      <c r="A108" s="1" t="inlineStr">
+    <row r="142" ht="22" customHeight="1">
+      <c r="A142" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>Steep Shaft  (가파른 샤프트)   ·   Club / Shaft / Angle/Plane · Steep</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="3" t="inlineStr">
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Steep Shaft  (가파른 샤프트)   ·   Shaft / Angle/Plane · Steep</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B109" s="4" t="inlineStr">
+      <c r="B143" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="22" customHeight="1">
-      <c r="A111" s="1" t="inlineStr">
+    <row r="145" ht="22" customHeight="1">
+      <c r="A145" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>Shallow Shaft  (눕는 샤프트)   ·   Club / Shaft / Angle/Plane · Shallow</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="3" t="inlineStr">
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Shallow Shaft  (눕는 샤프트)   ·   Shaft / Angle/Plane · Shallow</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B112" s="4" t="inlineStr">
+      <c r="B146" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="22" customHeight="1">
-      <c r="A114" s="1" t="inlineStr">
+    <row r="148" ht="22" customHeight="1">
+      <c r="A148" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>Casting  (캐스팅)   ·   Club / Club / Release · Cast</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="3" t="inlineStr">
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Casting  (캐스팅)   ·   Club / Release · Cast</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B115" s="4" t="inlineStr">
+      <c r="B149" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
@@ -3389,15 +3886,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -3418,15 +3914,10 @@
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Group(대분류)</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Object(소분류)</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -3450,15 +3941,10 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Rotation/Timing · Early
 [구분] pelvis_rotation_excessive (회전량); pelvis_stall (회전 속도)</t>
@@ -3483,15 +3969,10 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Rotation/Amount · Insufficient
 [구분] thorax_rotation_insufficient (분절이 다름)</t>
@@ -3516,15 +3997,10 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Rotation/Amount · Excessive
 [구분] spin_out (회전량+시퀀스 붕괴 복합); pelvis_open_early (타이밍)</t>
@@ -3549,15 +4025,10 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Rotation/Velocity · Stall
 [strong co-occur] handle_stall (선후 개인차, 양방향 연관 가능)</t>
@@ -3582,15 +4053,10 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Rotation/Amount · Insufficient</t>
         </is>
@@ -3614,15 +4080,10 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Rotation/Amount · Excessive</t>
         </is>
@@ -3646,15 +4107,10 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Rotation/Velocity · Stall
 [strong co-occur] pelvis_stall (선후 개인차)</t>
@@ -3679,15 +4135,10 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Rotation/Timing · Early
 [renamed from] Upper Body Open Early</t>
@@ -3712,15 +4163,10 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Pattern · Early Extension
 [role] Hub Node — 다수 원인이 모이고 다수 결과로 분기. In/Out-degree 모두 높음.</t>
@@ -3745,15 +4191,10 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
           <t>Spine</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Magnitude · Excessive
 [renamed from] Excessive Spine Extension
@@ -3779,15 +4220,10 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Position/Height (Vertical Axis) · Rise
 [role] Result Feature 성격 강함 — In-degree 높음.
@@ -3813,15 +4249,10 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Position/Height (Vertical Axis) · Drop
 [구분] head_elevation (단순 ± 관계 아님 — 원인·결과 Chain 상이)</t>
@@ -3846,15 +4277,10 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="inlineStr">
-        <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Position/Location (Horizontal Axis) · Trail
 [구분] hanging_back (체중 패턴)</t>
@@ -3879,15 +4305,10 @@
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Position/Height (Relative) · High</t>
         </is>
@@ -3911,15 +4332,10 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Position/Height (Relative) · Low</t>
         </is>
@@ -3943,15 +4359,10 @@
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Position/Depth · Deep
 [status] pending</t>
@@ -3976,15 +4387,10 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Position/Depth · Shallow
 [status] pending</t>
@@ -4009,15 +4415,10 @@
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Position/Direction · Forward
 [status] pending</t>
@@ -4042,15 +4443,10 @@
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Relationship · Far
 [status] pending</t>
@@ -4075,15 +4471,10 @@
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Relationship · Close
 [status] pending</t>
@@ -4108,15 +4499,10 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
           <t>Arm</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Timing · Late
 [status] pending</t>
@@ -4141,15 +4527,10 @@
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Upper Limb</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
           <t>Trail Elbow</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Location · Trail
 [status] pending</t>
@@ -4174,15 +4555,10 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
           <t>Shaft</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Angle/Plane · Steep
 [status] pending · referenced→feature 승격</t>
@@ -4207,15 +4583,10 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
           <t>Shaft</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Angle/Plane · Shallow
 [status] pending</t>
@@ -4243,12 +4614,7 @@
           <t>Club</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
-        <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Release · Cast
 [status] pending</t>
@@ -4273,15 +4639,10 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Location/Magnitude · Lead·Insufficient
 [status] pending · referenced→feature 승격</t>
@@ -4306,15 +4667,10 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>Location/Magnitude · Lead·Excessive
 [status] pending</t>
@@ -4339,15 +4695,10 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Timing · Late
 [status] pending</t>
@@ -4372,15 +4723,10 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Body</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Pattern · Spin-out
 [status] pending · referenced→feature 승격</t>
@@ -4388,7 +4734,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F30"/>
+  <autoFilter ref="A1:E30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4465,12 +4811,12 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Category Hierarchy</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Body{Pelvis·Thorax·Head·Spine·Pressure} / Upper Limb{Arm·Trail Elbow·Hands} / Club{Shaft·Club}</t>
+          <t>Object 단일 사용: Pelvis·Thorax·Head·Spine·Pressure·Arm·Trail Elbow·Hands·Shaft·Club  (규모 확대 시 Body/Upper Limb/Club 계층으로 확장 예정)</t>
         </is>
       </c>
     </row>
@@ -4897,14 +5243,14 @@
           <t>Pelvis Rotation Insufficient (골반 회전 부족)</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -4922,14 +5268,14 @@
           <t>Pelvis Rotation Excessive (골반 과회전)</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -4947,14 +5293,14 @@
           <t>Pelvis Stall (골반 회전 정지)</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(P6): Thorax 4종 표준화 + Category=Object·속성 태그화 (Phase 2)
Phase 1(구조) 종료, Phase 2(지식 축적) 시작. 구조 변경 없음.

Feature_Dictionary
- Category = Object 단일 기준 (Pelvis/Thorax/Pressure/Hands...)
- Rotation/Timing 등 속성은 비고에 태그로 이전 (예: "Rotation, Timing, Early")

P6 표준화 +4 (6섹션): Thorax Rotation Insufficient / Excessive / Stall / Open Early
→ 총 10/28 완료

Dictionary-first 준수 (기존 재사용 우선, 신규는 최소)
- 신규 Mechanism 2 (재사용 대상 함께 명시):
  · Backswing Coil Is Incomplete. (백스윙 코일 미완성 — Thorax Insuf/Stall, 향후 P4 재사용)
  · Rotational Power Transfer Decreases. (회전 에너지 전달 감소 — Loss of Power 링크)
- 나머지 Thorax 링크는 전부 기존 Mechanism 재사용 (M-ROT/PRS/ARM/CLB/CMP)
- Body Rotation Leads used_in에 pelvis_rotation_excessive 추가 (기존 Feature 재적용)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/DOH_Knowledge.xlsx
+++ b/DOH_Knowledge.xlsx
@@ -14,7 +14,7 @@
     <sheet name="TODO" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TODO'!$A$1:$E$29</definedName>
   </definedNames>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B149"/>
+  <dimension ref="A1:B197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1580,228 +1580,382 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 정의</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>Thorax Rotation Excessive  (흉곽 과회전)   ·   Thorax / Rotation/Amount · Excessive</t>
+          <t>다운스윙 중반(P6)에서 흉곽의 회전량이 정상보다 부족한 상태. 골반 회전과는 별개 Feature이며 상체 회전량(Amount) 부족이 핵심이다. Pelvis Rotation Insufficient와 강한 Co-occurrence이나 독립 유지한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient (P4, 백스윙 흉곽 회전 부족)
+   ↓
+Backswing Coil Is Incomplete.
+(백스윙 코일이 미완성된다.)
+   ↓
+Thorax Rotation Insufficient (흉곽 회전 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Insufficient (골반 회전 부족)
+   ↓
+Pelvis Rotation Does Not Complete Through Impact.
+(골반 회전이 임팩트까지 완성되지 않는다.)
+   ↓
+Thorax Rotation Insufficient (흉곽 회전 부족)</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A79" s="4" t="inlineStr"/>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="22" customHeight="1">
-      <c r="A81" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>Thorax Stall  (흉곽 회전 정지)   ·   Thorax / Rotation/Velocity · Stall</t>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+Pelvis Rotation Decelerates Before Impact.
+(임팩트 전에 골반 회전이 감속한다.)
+   ↓
+Thorax Rotation Insufficient (흉곽 회전 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr"/>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+Thorax Rotation Insufficient (흉곽 회전 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr"/>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+Pressure Remains On The Trail Side.
+(압력이 트레일측에 남아있다.)
+   ↓
+Thorax Rotation Insufficient (흉곽 회전 부족)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="22" customHeight="1">
-      <c r="A84" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>Thorax Open Early  (흉곽 조기 오픈)   ·   Thorax / Rotation/Timing · Early</t>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+Arm Delivery Space Is Reduced.
+(팔이 내려올 공간이 감소한다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr"/>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+Thorax Rotation Does Not Complete Through Impact.
+(흉곽 회전이 임팩트까지 완성되지 않는다.)
+   ↓
+Handle Stall (핸들 정지)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr"/>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+The Arms Compensate For Delayed Body Motion.
+(몸의 지연을 팔이 보상한다.)
+   ↓
+Casting (캐스팅)</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A85" s="4" t="inlineStr"/>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="22" customHeight="1">
-      <c r="A87" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>Spine Extension Excessive  (척추 과신전)   ·   Spine / Magnitude · Excessive</t>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr"/>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+Rotational Power Transfer Decreases.
+(회전 에너지 전달이 감소한다.)
+   ↓
+Loss of Power (파워 손실)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Rotation Insufficient (골반 회전 부족) — 강한 동반, 독립 축 유지
+· Pelvis Stall (골반 회전 정지)
+· Arm Stuck (팔 끼임)
+· Late Release (늦은 릴리즈)
+· Flip Release (플립 릴리즈)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 추가 검증 포인트</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="22" customHeight="1">
-      <c r="A90" s="1" t="inlineStr">
+          <t>· Thorax Rotation Insufficient와 Handle Stall이 높은 빈도로 함께 나타나는지 검증.
+· 회전 부족 골퍼의 Subtype: 팔 사용 증가(Casting) vs 회전 정지 동반(Pelvis/Thorax Stall).
+· 흉곽 회전 부족 → Club Face Open 빈도와 Flip Release 빈도 비교로 보상 패턴 세분화.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>· 흉곽 3축(Amount/Timing/Velocity) 중 Amount 축. 다운스윙에서는 '흉곽이 골반을 언제 얼마나 따라오는가'가 중요 → Open Early / Stall / Insufficient를 함께 분석.
+· 신규 표준 'Backswing Coil Is Incomplete.'는 P4 백스윙 기원 링크로, 향후 P4 시트의 백스윙 Feature에도 재사용한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>Head Elevation  (머리 상승)   ·   Head / Position/Height · Rise</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B91" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>Head Drop  (머리 하강)   ·   Head / Position/Height · Drop</t>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Excessive  (흉곽 과회전)   ·   Thorax / Rotation/Amount · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽의 회전량이 정상보다 과도한 상태. 회전 타이밍이 아니라 회전량(Amount)이 핵심이다. Pelvis와 동일하게 Amount/Timing/Velocity 축으로 분리 관리한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
+   ↓
+The Thorax Opens Before Arm Delivery.
+(팔 전달 전에 흉곽이 먼저 열린다.)
+   ↓
+Thorax Rotation Excessive (흉곽 과회전)</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A94" s="4" t="inlineStr"/>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="22" customHeight="1">
-      <c r="A96" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>Head Hanging Back  (머리 뒤잔류)   ·   Head / Position/Location · Trail</t>
+          <t>Pelvis Rotation Excessive (골반 과회전)
+   ↓
+Body Rotation Leads The Downswing.
+(몸통 회전이 다운스윙을 주도한다.)
+   ↓
+Thorax Rotation Excessive (흉곽 과회전)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr"/>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Open Early (골반 조기 오픈)
+   ↓
+The Pelvis Opens Before Arm Delivery.
+(팔 전달 전에 골반이 먼저 열린다.)
+   ↓
+Thorax Rotation Excessive (흉곽 과회전)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr"/>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Body Rotation Dominant (몸통 회전 주도)
+   ↓
+Body Rotation Leads The Downswing.
+(몸통 회전이 다운스윙을 주도한다.)
+   ↓
+Thorax Rotation Excessive (흉곽 과회전)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="22" customHeight="1">
-      <c r="A99" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>Lead Pressure Insufficient  (리드측 압력 부족)   ·   Pressure / Location/Magnitude · Lead·Insufficient</t>
+          <t>Thorax Rotation Excessive (흉곽 과회전)
+   ↓
+Thorax Rotation Outpaces Arm Delivery.
+(흉곽 회전이 팔 전달보다 앞선다.)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr"/>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Excessive (흉곽 과회전)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Arm Stuck (팔 끼임)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr"/>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Excessive (흉곽 과회전)
+   ↓
+The Body Rotates Around The Trail Side.
+(몸이 트레일측을 중심으로 회전한다.)
+   ↓
+Spin-out (스핀아웃)</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A100" s="4" t="inlineStr"/>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>Lead Pressure Excessive  (리드측 압력 과다)   ·   Pressure / Location/Magnitude · Lead·Excessive</t>
+          <t>Thorax Rotation Excessive (흉곽 과회전)
+   ↓
+The Club Approaches From Outside.
+(클럽이 바깥쪽 경로로 접근한다.)
+   ↓
+Outside Delivery (아웃사이드 딜리버리)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Rotation Excessive (골반 과회전)
+· Pelvis Open Early (골반 조기 오픈)
+· Thorax Open Early (흉곽 조기 오픈)
+· Club Face Open (클럽페이스 오픈)
+· Spin-out (스핀아웃)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>· Thorax Rotation Excessive와 Thorax Open Early는 자주 함께 나타나지만, 회전량은 많아도 오픈 타이밍은 정상인 골퍼 존재 여부.
+· Spin-out으로 이어지는 것이 회전량 자체 때문인지 골반 과회전 동시 발생 때문인지 검증.
+· Outside Delivery가 흉곽 과회전만으로도 발생하는 독립 패턴인지 확인.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 사고확장</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+          <t>· 흉곽 3축 중 Amount 축. Pelvis와 완전히 동일한 축 대응(Amount/Timing/Velocity) → AI가 두 분절을 동일 로직으로 분석 가능.
+· 'Upper Body Open Early' → 'Thorax Open Early' 통일로 해부학 객체명 일관성 확보.</t>
         </is>
       </c>
     </row>
@@ -1813,66 +1967,78 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Incomplete Pressure Transfer  (압력 이동 미완성)   ·   Pressure / Timing · Late</t>
+          <t>Thorax Stall  (흉곽 회전 정지)   ·   Thorax / Rotation/Velocity · Stall</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 정의</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="22" customHeight="1">
-      <c r="A108" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>High Hands  (손 높음)   ·   Hands / Position/Height · High (Relative)</t>
+          <t>다운스윙 중반(P6)에서 흉곽 회전이 정상보다 일찍 감속하거나 정지하는 현상. 회전량이 아니라 회전 속도(Velocity) 유지 실패가 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+Pelvis Rotation Decelerates Before Impact.
+(임팩트 전에 골반 회전이 감속한다.)
+   ↓
+Thorax Stall (흉곽 회전 정지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr"/>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Thorax Stall (흉곽 회전 정지)</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="3" t="inlineStr">
-        <is>
-          <t>■ 정의</t>
-        </is>
-      </c>
+      <c r="A109" s="4" t="inlineStr"/>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 높은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 충분히 하강하지 못한 상대 위치가 핵심이다.</t>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+Pressure Remains On The Trail Side.
+(압력이 트레일측에 남아있다.)
+   ↓
+Thorax Stall (흉곽 회전 정지)</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="inlineStr">
-        <is>
-          <t>■ 원인 추정</t>
-        </is>
-      </c>
+      <c r="A110" s="4" t="inlineStr"/>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Arm Depth Excessive (P4, 백스윙 손 과도한 깊이)
-   ↓
-The Hands Start Downswing From Behind The Thorax.
-(손이 몸통보다 뒤쪽에서 다운스윙을 시작한다.)
-   ↓
-The Thorax Rotates Rapidly During Transition.
-(전환 구간에서 흉곽이 급격하게 회전한다.)
-   ↓
-Rapid Thorax Rotation Reduces Available Arm Drop Time.
-(급격한 흉곽 회전으로 팔이 하강할 시간이 부족해진다.)
-   ↓
-High Hands (손 높음)</t>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Thorax Stall (흉곽 회전 정지)</t>
         </is>
       </c>
     </row>
@@ -1880,42 +2046,49 @@
       <c r="A111" s="4" t="inlineStr"/>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Arm Drop Insufficient (팔 하강 부족)
-   ↓
-Vertical Arm Drop During Downswing Is Insufficient.
-(다운스윙 동안 팔의 수직 하강이 충분하지 않다.)
-   ↓
-High Hands (손 높음)</t>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+Thorax Rotation Does Not Complete Through Impact.
+(흉곽 회전이 임팩트까지 완성되지 않는다.)
+   ↓
+Thorax Stall (흉곽 회전 정지)</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="4" t="inlineStr"/>
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Early Extension (얼리 익스텐션)
-   ↓
-The Body Loses Delivery Space.
-(다운스윙 공간이 부족해진다.)
-   ↓
-High Hands (손 높음)</t>
+          <t>Thorax Stall (흉곽 회전 정지)
+   ↓
+Thorax Rotation Decelerates Before Impact.
+(임팩트 전에 흉곽 회전이 감속한다.)
+   ↓
+Handle Stall (핸들 정지)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>■ 이후 나타날 가능성</t>
-        </is>
-      </c>
+      <c r="A113" s="4" t="inlineStr"/>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>High Hands (손 높음)
-   ↓
-The Club Approaches From A Steeper Delivery Pattern.
-(클럽이 가파른 전달 패턴으로 접근한다.)
-   ↓
-Steep Shaft (가파른 샤프트)</t>
+          <t>Thorax Stall (흉곽 회전 정지)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Late Release (늦은 릴리즈)</t>
         </is>
       </c>
     </row>
@@ -1923,12 +2096,12 @@
       <c r="A114" s="4" t="inlineStr"/>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>High Hands (손 높음)
-   ↓
-The Club Face Cannot Square In Time.
-(클럽페이스가 제시간에 스퀘어되지 못한다.)
-   ↓
-Club Face Open (클럽페이스 오픈)</t>
+          <t>Thorax Stall (흉곽 회전 정지)
+   ↓
+The Arms Compensate For Delayed Body Motion.
+(몸의 지연을 팔이 보상한다.)
+   ↓
+Casting (캐스팅)</t>
         </is>
       </c>
     </row>
@@ -1936,22 +2109,189 @@
       <c r="A115" s="4" t="inlineStr"/>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>High Hands (손 높음)
+          <t>Thorax Stall (흉곽 회전 정지)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈) / Club Face Closed (클럽페이스 클로즈)  ※보상 방식에 따라</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Stall (골반 회전 정지) — 선후 개인차, 강한 동반
+· Handle Stall (핸들 정지)
+· Flip Release (플립 릴리즈)
+· Arm Stuck (팔 끼임)
+· Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Stall과 Thorax Stall 중 어느 쪽이 먼저 발생하는 경우가 많은지 검증.
+· Thorax Stall 이후 Casting vs Handle Stall→Flip 보상 경향 Subtype 분석.
+· 완전 정지 유형 vs 단순 감속 유형 세분 필요성 검토.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>· 흉곽 3축 중 Velocity 축. Pelvis Stall과 Thorax Stall은 강한 Co-occurrence이나 골반만/흉곽만 멈추는 유형이 모두 존재 → 독립 Feature 유지.
+· Stall 계열은 'Handle Stall → Flip Release' 결과 경로를 공통 표준으로 재사용한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Thorax Open Early  (흉곽 조기 오픈)   ·   Thorax / Rotation/Timing · Early</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽이 정상보다 이른 타이밍에 목표 방향으로 열리는 현상. 회전량이 아니라 회전 시점(Timing)이 빠른 것이 핵심이다. (Upper Body Open Early에서 명명 통일)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Open Early (골반 조기 오픈)
+   ↓
+The Pelvis Opens Before Arm Delivery.
+(팔 전달 전에 골반이 먼저 열린다.)
+   ↓
+Thorax Open Early (흉곽 조기 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr"/>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Body Rotation Dominant (몸통 회전 주도)
+   ↓
+Body Rotation Leads The Downswing.
+(몸통 회전이 다운스윙을 주도한다.)
+   ↓
+Thorax Open Early (흉곽 조기 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr"/>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Arm Drop Insufficient (팔 하강 부족)
+   ↓
+Arm Drop Is Insufficient.
+(팔의 하강이 충분하지 않다.)
+   ↓
+Thorax Open Early (흉곽 조기 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr"/>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
+Thorax Open Early (흉곽 조기 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
+   ↓
+The Club Approaches From A Steeper Delivery Pattern.
+(클럽이 가파른 전달 패턴으로 접근한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr"/>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
+   ↓
+Thorax Rotation Outpaces Arm Delivery.
+(흉곽 회전이 팔 전달보다 앞선다.)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr"/>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
    ↓
 The Arms Fall Behind The Rotating Body.
 (회전하는 몸에 비해 팔이 뒤처진다.)
    ↓
-Arm Stuck (팔 끼임)
-   ↓
-Late Release (늦은 릴리즈)</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="4" t="inlineStr"/>
-      <c r="B116" s="4" t="inlineStr">
-        <is>
-          <t>High Hands (손 높음)
+Arm Stuck (팔 끼임)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr"/>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
    ↓
 The Club Approaches From Outside.
 (클럽이 바깥쪽 경로로 접근한다.)
@@ -1960,13 +2300,367 @@
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="3" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="4" t="inlineStr"/>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
+   ↓
+The Body Rotates Around The Trail Side.
+(몸이 트레일측을 중심으로 회전한다.)
+   ↓
+Spin-out (스핀아웃)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
         <is>
           <t>■ Strong Co-occurrence</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr">
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>· Pelvis Open Early (골반 조기 오픈) — 상·하체 동시 조기 오픈
+· Club Face Open (클럽페이스 오픈)
+· Steep Shaft (가파른 샤프트)
+· Outside Delivery (아웃사이드 딜리버리)
+· Spin-out (스핀아웃)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>· Thorax Open Early와 Pelvis Open Early가 항상 함께인지, 상체만 먼저 열리는 Subtype이 얼마나 존재하는지.
+· Thorax Open Early가 Steep Shaft 없이도 Outside Delivery로 이어지는 사례 확인.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>· 흉곽 3축 중 Timing 축. Pelvis와 Thorax가 Amount/Timing/Velocity 6칸 완전 대응 → 동일 로직 분석.
+· Upper Body 용어를 프로젝트 전체에서 폐기하고 Head/Thorax/Pelvis/Arm/Hand/Shaft/Club Face/Pressure 등 해부학·명확 객체명으로 통일.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Spine Extension Excessive  (척추 과신전)   ·   Spine / Magnitude · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Head Elevation  (머리 상승)   ·   Head / Position/Height · Rise</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="22" customHeight="1">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Head Drop  (머리 하강)   ·   Head / Position/Height · Drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Head Hanging Back  (머리 뒤잔류)   ·   Head / Position/Location · Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="22" customHeight="1">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient  (리드측 압력 부족)   ·   Pressure / Location/Magnitude · Lead·Insufficient</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="22" customHeight="1">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive  (리드측 압력 과다)   ·   Pressure / Location/Magnitude · Lead·Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="22" customHeight="1">
+      <c r="A153" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Incomplete Pressure Transfer  (압력 이동 미완성)   ·   Pressure / Timing · Late</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>(상태)</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="22" customHeight="1">
+      <c r="A156" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>High Hands  (손 높음)   ·   Hands / Position/Height · High (Relative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 높은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 충분히 하강하지 못한 상대 위치가 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>Arm Depth Excessive (P4, 백스윙 손 과도한 깊이)
+   ↓
+The Hands Start Downswing From Behind The Thorax.
+(손이 몸통보다 뒤쪽에서 다운스윙을 시작한다.)
+   ↓
+The Thorax Rotates Rapidly During Transition.
+(전환 구간에서 흉곽이 급격하게 회전한다.)
+   ↓
+Rapid Thorax Rotation Reduces Available Arm Drop Time.
+(급격한 흉곽 회전으로 팔이 하강할 시간이 부족해진다.)
+   ↓
+High Hands (손 높음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr"/>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>Arm Drop Insufficient (팔 하강 부족)
+   ↓
+Vertical Arm Drop During Downswing Is Insufficient.
+(다운스윙 동안 팔의 수직 하강이 충분하지 않다.)
+   ↓
+High Hands (손 높음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr"/>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Body Loses Delivery Space.
+(다운스윙 공간이 부족해진다.)
+   ↓
+High Hands (손 높음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>High Hands (손 높음)
+   ↓
+The Club Approaches From A Steeper Delivery Pattern.
+(클럽이 가파른 전달 패턴으로 접근한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr"/>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>High Hands (손 높음)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr"/>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>High Hands (손 높음)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="4" t="inlineStr"/>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>High Hands (손 높음)
+   ↓
+The Club Approaches From Outside.
+(클럽이 바깥쪽 경로로 접근한다.)
+   ↓
+Outside Delivery (아웃사이드 딜리버리)</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B165" s="4" t="inlineStr">
         <is>
           <t>· Steep Shaft (가파른 샤프트)
 · Handle Raise (핸들 상승)
@@ -1975,267 +2669,267 @@
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="3" t="inlineStr">
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
         <is>
           <t>■ 추가 검증 포인트</t>
         </is>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B166" s="4" t="inlineStr">
         <is>
           <t>· High Hands가 '손이 높아서'인지 '몸의 회전에 비해 손이 늦게 내려와서'인지 레슨 데이터로 구분 필요 (후자 가능성 높음).
 · High Hands → Steep Shaft는 흔한 조합이나, 높은 손에서도 샤프트를 눕혀 전달하는 예외 골퍼 존재 여부 확인.</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="3" t="inlineStr">
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
         <is>
           <t>■ 사고확장</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B167" s="4" t="inlineStr">
         <is>
           <t>· P6 손 위치 Feature는 모두 상대 위치(Relative Position): '이 시점의 다운스윙 진행에서 정상이라면 손이 어디 있어야 하는가' 기준. High/Low/Deep/Shallow 전부 동일 철학.
 · High Hands는 P4→Transition→P6를 잇는 Cross-Phase Chain의 대표 사례. P7 Steep Shaft/Outside Delivery로 이어진다.</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="22" customHeight="1">
-      <c r="A121" s="1" t="inlineStr">
+    <row r="169" ht="22" customHeight="1">
+      <c r="A169" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B121" s="2" t="inlineStr">
+      <c r="B169" s="2" t="inlineStr">
         <is>
           <t>Low Hands  (손 낮음)   ·   Hands / Position/Height · Low (Relative)</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="3" t="inlineStr">
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="B170" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="22" customHeight="1">
-      <c r="A124" s="1" t="inlineStr">
+    <row r="172" ht="22" customHeight="1">
+      <c r="A172" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B124" s="2" t="inlineStr">
+      <c r="B172" s="2" t="inlineStr">
         <is>
           <t>Deep Hands  (손 깊음)   ·   Hands / Position/Depth · Deep</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" s="3" t="inlineStr">
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B125" s="4" t="inlineStr">
+      <c r="B173" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="22" customHeight="1">
-      <c r="A127" s="1" t="inlineStr">
+    <row r="175" ht="22" customHeight="1">
+      <c r="A175" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B127" s="2" t="inlineStr">
+      <c r="B175" s="2" t="inlineStr">
         <is>
           <t>Forward Hands  (손 전방)   ·   Hands / Position/Direction · Forward</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="3" t="inlineStr">
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B128" s="4" t="inlineStr">
+      <c r="B176" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="22" customHeight="1">
-      <c r="A130" s="1" t="inlineStr">
+    <row r="178" ht="22" customHeight="1">
+      <c r="A178" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B130" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Hands Too Far From Body  (손이 몸에서 멀어짐)   ·   Hands / Relationship · Far</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="3" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B131" s="4" t="inlineStr">
+      <c r="B179" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="22" customHeight="1">
-      <c r="A133" s="1" t="inlineStr">
+    <row r="181" ht="22" customHeight="1">
+      <c r="A181" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B133" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Hands Too Close To Body  (손이 몸에 가까움)   ·   Hands / Relationship · Close</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="3" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B134" s="4" t="inlineStr">
+      <c r="B182" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="22" customHeight="1">
-      <c r="A136" s="1" t="inlineStr">
+    <row r="184" ht="22" customHeight="1">
+      <c r="A184" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Late Arm  (팔 하강 지연)   ·   Arm / Timing · Late</t>
         </is>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="3" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B137" s="4" t="inlineStr">
+      <c r="B185" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="22" customHeight="1">
-      <c r="A139" s="1" t="inlineStr">
+    <row r="187" ht="22" customHeight="1">
+      <c r="A187" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B139" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Trail Elbow Behind Body  (트레일 팔꿈치 뒤처짐)   ·   Trail Elbow / Location · Trail</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" s="3" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B140" s="4" t="inlineStr">
+      <c r="B188" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="142" ht="22" customHeight="1">
-      <c r="A142" s="1" t="inlineStr">
+    <row r="190" ht="22" customHeight="1">
+      <c r="A190" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Steep Shaft  (가파른 샤프트)   ·   Shaft / Angle/Plane · Steep</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="3" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B143" s="4" t="inlineStr">
+      <c r="B191" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="22" customHeight="1">
-      <c r="A145" s="1" t="inlineStr">
+    <row r="193" ht="22" customHeight="1">
+      <c r="A193" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B145" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Shallow Shaft  (눕는 샤프트)   ·   Shaft / Angle/Plane · Shallow</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="3" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B146" s="4" t="inlineStr">
+      <c r="B194" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="22" customHeight="1">
-      <c r="A148" s="1" t="inlineStr">
+    <row r="196" ht="22" customHeight="1">
+      <c r="A196" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B148" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Casting  (캐스팅)   ·   Club / Release · Cast</t>
         </is>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="3" t="inlineStr">
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B149" s="4" t="inlineStr">
+      <c r="B197" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
@@ -2252,7 +2946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2303,169 +2997,237 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
+          <t>Backswing Coil Is Incomplete.</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>백스윙 코일이 미완성된다.</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Backswing Thorax Rotation Insufficient
+Incomplete Coil</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>thorax_rotation_insufficient
+thorax_stall</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>P6 리팩토링 중 신규 (2026-07-07). P4 백스윙 기원 — 흉곽 회전 부족/정지 상류 링크. (기존 Feature 재적용 검토: 향후 P4 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
           <t>Body Rotation Leads The Downswing.</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>몸통 회전이 다운스윙을 주도한다.</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Body Rotation Dominant
 Upper Body Dominance</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early
 thorax_open_early
-thorax_rotation_excessive</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
+thorax_rotation_excessive
+pelvis_rotation_excessive</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>P6 리팩토링 중 신규 (2026-07-07)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Pelvis Rotation Decelerates Before Impact.</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>임팩트 전에 골반 회전이 감속한다.</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Pelvis Rotation Stops
 The Hips Stall
 Pelvis Slows Down Early</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>pelvis_stall</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Pelvis Rotation Does Not Complete Through Impact.</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>골반 회전이 임팩트까지 완성되지 않는다.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Insufficient Pelvis Rotation
 The Hips Do Not Turn Enough</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>pelvis_rotation_insufficient</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Rotational Power Transfer Decreases.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>회전 에너지 전달이 감소한다.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Loss Of Rotational Power
+Energy Transfer Drops</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>thorax_rotation_insufficient</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>P6 리팩토링 중 신규 (2026-07-07). Loss of Power 결과 링크.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>The Body Rotates Around The Trail Side.</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>몸이 트레일측을 중심으로 회전한다.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>The Body Spins Around The Right Side
 Rotation Axis Stays On The Trail Side</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>spin_out
 pelvis_rotation_excessive</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>The Lead Side Cannot Become The Primary Rotation Axis.</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>리드측이 주 회전축이 되지 못한다.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>The Body Cannot Rotate Around The Lead Side Efficiently
 No Left Side Post</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>pelvis_stall
 early_extension</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>The Pelvis Opens Before Arm Delivery.</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>팔 전달 전에 골반이 먼저 열린다.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>The Pelvis Opens Early
 The Pelvis Opens Too Soon
@@ -2475,256 +3237,256 @@
 The Body Opens Early</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>The Pelvis Rotates Faster Than The Arms Can Follow.</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>팔이 따라올 수 없을 만큼 골반이 빠르게 회전한다.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>The Hips Outrun The Arms
 Pelvis Outpaces Arm Delivery</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>pelvis_rotation_excessive</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>The Thorax Opens Before Arm Delivery.</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>팔 전달 전에 흉곽이 먼저 열린다.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>The Upper Body Opens Early
 The Thorax Opens Too Soon
 The Chest Opens Early</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>thorax_open_early
 thorax_rotation_excessive</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>The Thorax Rotates Rapidly During Transition.</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>전환 구간에서 흉곽이 급격하게 회전한다.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Rapid Thorax Rotation
 The Thorax Spins Fast Early</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>high_hands
 arm_stuck</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>M001~M007 시트의 Rapid Thorax Rotation 표준화.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Thorax Rotation Decelerates Before Impact.</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>임팩트 전에 흉곽 회전이 감속한다.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Thorax Rotation Stops
 The Chest Stalls</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>thorax_stall</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Thorax Rotation Does Not Complete Through Impact.</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>흉곽 회전이 임팩트까지 완성되지 않는다.</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Insufficient Thorax Rotation
 The Chest Does Not Turn Enough</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>thorax_rotation_insufficient</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Thorax Rotation Is Delayed.</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>흉곽 회전이 지연된다.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Thorax Rotation Lags
 The Chest Turns Late</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>thorax_rotation_insufficient</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>시트 M004.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>ROT</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Trail Leg Drive Opens The Pelvis Early.</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>트레일 다리의 추진이 골반을 조기에 연다.</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Trail Leg Push Early
 Trail Leg Push Excessive</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early
 pelvis_rotation_excessive</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>P6 리팩토링 중 신규 (2026-07-07)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>PRS</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Pressure Does Not Reach The Lead Side Before Impact.</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>임팩트 전까지 압력이 리드측에 도달하지 못한다.</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Late Pressure Shift
 Lead Side Pressure Insufficient
 Weight Does Not Get Left In Time</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>pelvis_rotation_insufficient
 pelvis_stall
@@ -2734,84 +3496,84 @@
 spine_extension_excessive</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>PRS</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Pressure On The Lead Side Becomes Excessive.</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>리드측 압력이 과도해진다.</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Excessive
 Too Much Weight Left</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>pelvis_rotation_excessive
 head_drop</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>PRS</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Pressure Remains On The Lead Side.</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>압력이 리드측에 남아있다.</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Weight Stuck On Left
 Reverse Pivot Pressure</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>백스윙 리드측 압력 잔류(Reverse Pivot) 표현. P4~P5 연계용으로 예약.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>PRS</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Pressure Remains On The Trail Side.</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>압력이 트레일측에 남아있다.</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Pressure Stays On The Right Side
 Weight Remains On The Trail Side
@@ -2819,565 +3581,565 @@
 Hanging Back Pressure</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>hanging_back
 head_hanging_back</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>PRS</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Pressure Transfers To The Lead Side Too Early.</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>압력이 리드측으로 너무 빨리 이동한다.</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Early
 Early Weight Shift Left
 Pressure Moves Left Too Soon</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early
 lead_pressure_excessive</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>PRS</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>The Player Never Establishes Adequate Trail Side Loading.</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>충분한 트레일측 하중이 형성되지 않는다.</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>No Trail Side Load
 Trail Loading Failure
 Weak Backswing Load</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>hanging_back</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Reverse Pivot 상위 경로와 연결 (Node Library N03).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Arm Delivery Space Is Reduced.</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>팔이 내려올 공간이 감소한다.</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Less Room For The Arms
 Arm Space Shrinks</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early
 early_extension
 arm_drop_insufficient</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Arm Drop Is Insufficient.</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>팔의 하강이 충분하지 않다.</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Arms Do Not Drop Enough
 Arm Drop Insufficient</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>high_hands
 steep_shaft
 arm_drop_insufficient</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>시트 Mechanism (Arm Drop Is Insufficient).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Rapid Thorax Rotation Reduces Available Arm Drop Time.</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>급격한 흉곽 회전으로 팔이 하강할 시간이 부족해진다.</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>No Time For Arms To Drop
 Fast Chest Leaves No Arm Time</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>high_hands</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>P4→P6 연결 체인의 핵심 Transition Mechanism.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>The Arm Starts Downswing From A Higher Position.</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>팔이 높은 위치에서 다운스윙을 시작한다.</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Arms High At Transition
 Arm Starts Downswing From Higher Position</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>high_hands</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>시트 M001.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>The Arms Cannot Reach Delivery Position In Time.</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>팔이 전달 위치에 제시간에 도달하지 못한다.</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>The Arms Are Late
 Arms Cannot Catch Up</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>late_release
 arm_drop_insufficient</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>The Arms Fall Behind The Rotating Body.</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>회전하는 몸에 비해 팔이 뒤처진다.</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>The Arms Get Stuck Behind
 Arm Stuck
 The Arms Trail The Body</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>arm_stuck
 pelvis_rotation_excessive
 thorax_rotation_excessive</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>The Hands Start Downswing From Behind The Thorax.</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>손이 몸통보다 뒤쪽에서 다운스윙을 시작한다.</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Hands Behind The Body At Transition
 Hands Trapped Behind</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>high_hands</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>시트 M003. P4 Arm Depth Excessive → P6 High Hands 체인의 시작 링크.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>The Trail Elbow Falls Behind The Thorax.</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>트레일 팔꿈치가 흉곽보다 뒤처진다.</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Trail Elbow Stuck
 Right Elbow Behind Body</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Thorax Rotation Outpaces Arm Delivery.</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>흉곽 회전이 팔 전달보다 앞선다.</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>The Chest Beats The Arms
 Body Ahead Of Arms</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>thorax_open_early
 thorax_rotation_excessive</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Vertical Arm Drop During Downswing Is Insufficient.</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>다운스윙 동안 팔의 수직 하강이 충분하지 않다.</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Insufficient Vertical Arm Drop During Downswing</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>high_hands
 steep_shaft</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>시트 M002. M-ARM-06의 수직 방향 특화 변형.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Lag Is Lost Before Impact.</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>임팩트 전에 래그가 소실된다.</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Loss Of Lag
 Angle Released Too Soon</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>The Club Approaches From A Steeper Delivery Pattern.</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>클럽이 가파른 전달 패턴으로 접근한다.</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Steep Shaft Delivery
 The Shaft Steepens</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>steep_shaft
 high_hands</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>The Club Approaches From Outside.</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>클럽이 바깥쪽 경로로 접근한다.</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Over The Top
 Outside Delivery
 Out-To-In Path</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>outside_delivery</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>The Club Bottoms Out Behind The Ball.</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>클럽 최저점이 볼 뒤에서 형성된다.</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>Low Point Behind Ball
 Bottoms Out Early</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>fat_contact
 head_drop
 head_hanging_back</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>The Club Face Cannot Square In Time.</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>클럽페이스가 제시간에 스퀘어되지 못한다.</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>Face Stays Open
 Face Cannot Rotate In Time</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>club_face_open</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>The Club Is Released Early To Reach The Ball.</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>공에 도달하기 위해 클럽을 조기에 푼다.</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Casting
 Early Release
@@ -3385,497 +4147,497 @@
 Hand Dominance Release</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>The Clubhead Overtakes The Hands Early.</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>클럽헤드가 손보다 먼저 앞선다.</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>Flip
 Clubhead Passes Hands Early
 Scoop</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>flip_release</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Reduced Arm Space Promotes Early Club Release.</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>팔 공간 부족으로 클럽을 조기에 풀게 된다.</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>No Space Forces Casting
 Tight Space Causes Early Release</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>casting
 early_extension</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>The Body Loses Delivery Space.</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>다운스윙 공간이 부족해진다.</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>No Room To Deliver
 Space Collapses</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>early_extension
 high_hands</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>The Body Moves Toward The Ball And Loses Space.</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>몸이 볼 방향으로 이동하며 공간을 잃는다.</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Body Drifts To The Ball
 Toward-Ball Movement</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>early_extension
 high_hands</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>The Body Reaches The Lead Side Before The Arms.</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>몸이 팔보다 먼저 리드측에 도달한다.</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>Body Ahead Of Arms Into Impact
 Body Gets Left First</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early
 arm_stuck</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>The Lead Arm Remains Connected To The Thorax.</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>리드암이 흉곽에 계속 붙어 있다.</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>Lead Arm Trapped On Chest
 No Arm Separation</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>The Lead Hip Cannot Accept Body Load.</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>리드 고관절이 하중을 받아들이지 못한다.</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>Lead Hip Fails To Load
 No Left Hip Acceptance</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>early_extension
 pelvis_stall</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>The Lead Leg Accepts Body Load Too Early.</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>리드다리가 너무 일찍 하중을 받아낸다.</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Early Lead Leg Load
 Left Leg Loads Too Soon</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>The Lead Side Cannot Stabilize During Transition.</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>전환 과정에서 리드측이 안정되지 못한다.</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>Lead Side Collapses
 No Left Side Stability</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>early_extension</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>The Trail Side Continues Supporting Rotation.</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>트레일측이 계속 회전을 지지한다.</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>Trail Side Keeps Posting
 Right Side Stays Loaded</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>hanging_back
 head_hanging_back</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>The Arms Compensate For Delayed Body Motion.</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>몸의 지연을 팔이 보상한다.</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Arms Save The Swing
 Arm Compensation</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release
 arm_stuck</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="12" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>The Body Extends Early To Create Space.</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>공간을 만들기 위해 몸이 일찍 신전한다.</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>Stand Up To Make Room
 Early Extension Compensation</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>early_extension
 spine_extension_excessive
 head_elevation</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="12" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>The Hands Take Over Club Delivery.</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>손이 클럽 전달을 주도한다.</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>Hand Dominance Increase
 Hands Take Control</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>flip_release
 casting
 hand_dominance_increase</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="12" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>The Lead Arm Separates From The Thorax.</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>리드암이 몸통과 분리된다.</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>Chicken Wing
 Lead Arm Flies Off Chest</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>시트 M007. Chicken Wing 전조. P7 연계용 예약.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>The Trail Arm Extends Early To Deliver The Club.</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>클럽 전달을 위해 트레일 팔이 일찍 펴진다.</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>Right Arm Straightens Early
 Early Trail Arm Extension</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>casting</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="12" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>The Trail Elbow Collapses Toward The Body.</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>트레일 팔꿈치가 몸통 쪽으로 급격하게 붙는다.</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>Trail Elbow Pinch
 Right Elbow Jams In</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>시트 M006.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F52"/>
+  <autoFilter ref="A1:F54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3946,7 +4708,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Timing · Early
+          <t>Rotation, Timing, Early
 [구분] pelvis_rotation_excessive (회전량); pelvis_stall (회전 속도)</t>
         </is>
       </c>
@@ -3974,7 +4736,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Amount · Insufficient
+          <t>Rotation, Amount, Insufficient
 [구분] thorax_rotation_insufficient (분절이 다름)</t>
         </is>
       </c>
@@ -4002,7 +4764,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Amount · Excessive
+          <t>Rotation, Amount, Excessive
 [구분] spin_out (회전량+시퀀스 붕괴 복합); pelvis_open_early (타이밍)</t>
         </is>
       </c>
@@ -4030,7 +4792,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Velocity · Stall
+          <t>Rotation, Velocity, Stall
 [strong co-occur] handle_stall (선후 개인차, 양방향 연관 가능)</t>
         </is>
       </c>
@@ -4058,7 +4820,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Amount · Insufficient</t>
+          <t>Rotation, Amount, Insufficient</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4847,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Amount · Excessive</t>
+          <t>Rotation, Amount, Excessive</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4874,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Velocity · Stall
+          <t>Rotation, Velocity, Stall
 [strong co-occur] pelvis_stall (선후 개인차)</t>
         </is>
       </c>
@@ -4140,7 +4902,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Rotation/Timing · Early
+          <t>Rotation, Timing, Early
 [renamed from] Upper Body Open Early</t>
         </is>
       </c>
@@ -4168,7 +4930,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Pattern · Early Extension
+          <t>Pattern, Early Extension
 [role] Hub Node — 다수 원인이 모이고 다수 결과로 분기. In/Out-degree 모두 높음.</t>
         </is>
       </c>
@@ -4196,7 +4958,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Magnitude · Excessive
+          <t>Magnitude, Excessive
 [renamed from] Excessive Spine Extension
 [구분] early_extension (분절: 골반/고관절)</t>
         </is>
@@ -4225,7 +4987,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Position/Height (Vertical Axis) · Rise
+          <t>Position, Height, Rise
 [role] Result Feature 성격 강함 — In-degree 높음.
 [phase] P6에서는 초기 발생, P7에서 최종 관찰되는 경우가 많음. 두 구간 체크 대상.</t>
         </is>
@@ -4254,7 +5016,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Position/Height (Vertical Axis) · Drop
+          <t>Position, Height, Drop
 [구분] head_elevation (단순 ± 관계 아님 — 원인·결과 Chain 상이)</t>
         </is>
       </c>
@@ -4282,7 +5044,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Position/Location (Horizontal Axis) · Trail
+          <t>Position, Location, Trail
 [구분] hanging_back (체중 패턴)</t>
         </is>
       </c>
@@ -4310,7 +5072,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Position/Height (Relative) · High</t>
+          <t>Position, Height, High</t>
         </is>
       </c>
     </row>
@@ -4337,7 +5099,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Position/Height (Relative) · Low</t>
+          <t>Position, Height, Low</t>
         </is>
       </c>
     </row>
@@ -4364,7 +5126,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Position/Depth · Deep
+          <t>Position, Depth, Deep
 [status] pending</t>
         </is>
       </c>
@@ -4392,7 +5154,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Position/Depth · Shallow
+          <t>Position, Depth, Shallow
 [status] pending</t>
         </is>
       </c>
@@ -4420,7 +5182,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Position/Direction · Forward
+          <t>Position, Direction, Forward
 [status] pending</t>
         </is>
       </c>
@@ -4448,7 +5210,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Relationship · Far
+          <t>Relationship, Far
 [status] pending</t>
         </is>
       </c>
@@ -4476,7 +5238,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Relationship · Close
+          <t>Relationship, Close
 [status] pending</t>
         </is>
       </c>
@@ -4504,7 +5266,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Timing · Late
+          <t>Timing, Late
 [status] pending</t>
         </is>
       </c>
@@ -4532,7 +5294,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Location · Trail
+          <t>Location, Trail
 [status] pending</t>
         </is>
       </c>
@@ -4560,7 +5322,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Angle/Plane · Steep
+          <t>Angle, Plane, Steep
 [status] pending · referenced→feature 승격</t>
         </is>
       </c>
@@ -4588,7 +5350,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Angle/Plane · Shallow
+          <t>Angle, Plane, Shallow
 [status] pending</t>
         </is>
       </c>
@@ -4616,7 +5378,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Release · Cast
+          <t>Release, Cast
 [status] pending</t>
         </is>
       </c>
@@ -4644,7 +5406,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Location/Magnitude · Lead·Insufficient
+          <t>Location, Magnitude, Lead, Insufficient
 [status] pending · referenced→feature 승격</t>
         </is>
       </c>
@@ -4672,7 +5434,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Location/Magnitude · Lead·Excessive
+          <t>Location, Magnitude, Lead, Excessive
 [status] pending</t>
         </is>
       </c>
@@ -4700,7 +5462,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Timing · Late
+          <t>Timing, Late
 [status] pending</t>
         </is>
       </c>
@@ -4728,7 +5490,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Pattern · Spin-out
+          <t>Pattern, Spin-out
 [status] pending · referenced→feature 승격</t>
         </is>
       </c>
@@ -5368,14 +6130,14 @@
           <t>Thorax Rotation Insufficient (흉곽 회전 부족)</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -5393,14 +6155,14 @@
           <t>Thorax Rotation Excessive (흉곽 과회전)</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -5418,14 +6180,14 @@
           <t>Thorax Stall (흉곽 회전 정지)</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -5443,14 +6205,14 @@
           <t>Thorax Open Early (흉곽 조기 오픈)</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(P6): Head 3 + Spine 표준화 + Co-occurrence ★ 부여 연기(무등급 통일)
Phase 2-1(Feature 완성) 우선. ★ 등급은 전 Feature 완료 후 일괄.

P6 표준화 +4 (6섹션): Spine Extension Excessive / Head Elevation
  / Head Drop / Head Hanging Back  → 총 18/28 완료

Strong Co-occurrence 무등급 나열로 통일
- 앞서 Pressure/Spin-out에 넣었던 ★를 무등급 '· Feature'로 환원 (전 Feature 일관)
- Naming_Rule/TODO에 'Co-occurrence Review Day'(Phase 2-2) 명시 — 전 Feature 완료 후 ★ 일괄, 그날 Feature 수정 금지

Dictionary-first — Head/Spine 자세 도메인 확장
- 신규 Mechanism 7 (CMP 6·CLB 1) → 총 72
  · 상체 신전/굴곡·측굴·머리 상승/하강/트레일 잔류·회전축 상승 등 자세 링크
  · The Club Approaches From Inside. (M-CLB-02 Outside의 대응)
- 신규 Feature 5 (Spine Flexion Excessive, Trail Side Bend Excessive,
  Handle Raise, Handle Too Low, Spine Angle Loss) → 39
- 나머지 링크는 기존 Mechanism 재사용

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/DOH_Knowledge.xlsx
+++ b/DOH_Knowledge.xlsx
@@ -14,8 +14,8 @@
     <sheet name="TODO" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TODO'!$A$1:$E$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -162,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -223,6 +223,7 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -589,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B252"/>
+  <dimension ref="A1:B296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1536,12 +1537,12 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>★★★★★ Lead Pressure Insufficient (리드측 압력 부족)
-★★★★★ Incomplete Pressure Transfer (압력 이동 미완성)
-★★★★★ Hanging Back (체중 뒤잔류)
-★★★★☆ Late Arm (팔 하강 지연)
-★★★★☆ Outside Delivery (아웃사이드 딜리버리)
-★★★★☆ Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)</t>
+          <t>· Lead Pressure Insufficient (리드측 압력 부족)
+· Incomplete Pressure Transfer (압력 이동 미완성)
+· Hanging Back (체중 뒤잔류)
+· Late Arm (팔 하강 지연)
+· Outside Delivery (아웃사이드 딜리버리)
+· Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)</t>
         </is>
       </c>
     </row>
@@ -2564,138 +2565,194 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 정의</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="22" customHeight="1">
-      <c r="A152" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>Head Elevation  (머리 상승)   ·   Head / Position/Height · Rise</t>
+          <t>다운스윙 중반(P6)에서 척추(흉요추)가 정상보다 과도하게 신전되어 상체가 뒤로 젖는 현상. 평가 분절이 골반·고관절인 Early Extension과 구분한다 (척추·몸통).</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+The Torso Extends Backward To Recover Balance.
+(균형 회복을 위해 상체가 뒤로 신전한다.)
+   ↓
+Spine Extension Excessive (척추 과신전)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr"/>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+The Torso Extends Backward To Recover Balance.
+(균형 회복을 위해 상체가 뒤로 신전한다.)
+   ↓
+Spine Extension Excessive (척추 과신전)</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A153" s="4" t="inlineStr"/>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="22" customHeight="1">
-      <c r="A155" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
-        <is>
-          <t>Head Drop  (머리 하강)   ·   Head / Position/Height · Drop</t>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
+Spine Extension Excessive (척추 과신전)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>Spine Extension Excessive (척추 과신전)
+   ↓
+The Head Rises As The Body Stands Up.
+(몸이 일어나면서 머리가 상승한다.)
+   ↓
+Head Elevation (머리 상승)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr"/>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Spine Extension Excessive (척추 과신전)
+   ↓
+The Body Loses Delivery Space.
+(다운스윙 공간이 부족해진다.)
+   ↓
+Handle Raise (핸들 상승)</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A156" s="4" t="inlineStr"/>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="158" ht="22" customHeight="1">
-      <c r="A158" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>Head Hanging Back  (머리 뒤잔류)   ·   Head / Position/Location · Trail</t>
+          <t>Spine Extension Excessive (척추 과신전)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr"/>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Spine Extension Excessive (척추 과신전)
+   ↓
+The Club Approaches From A Steeper Delivery Pattern.
+(클럽이 가파른 전달 패턴으로 접근한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>· Head Elevation (머리 상승)
+· Early Extension (얼리 익스텐션)
+· Handle Raise (핸들 상승)
+· Hanging Back (체중 뒤잔류)
+· Club Face Open (클럽페이스 오픈)</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 추가 검증 포인트</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="161" ht="22" customHeight="1">
-      <c r="A161" s="1" t="inlineStr">
+          <t>· 허리만 과신전되고 골반은 비교적 유지되는 Spine Dominant Subtype이 얼마나 자주 나타나는지 확인.
+· Spine Extension Excessive가 항상 Head Elevation을 동반하는지, 목·머리는 유지한 채 흉요추만 신전되는 유형이 있는지 검증.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>· 평가 분절이 다르다: Early Extension → 골반·고관절 / Spine Extension Excessive → 척추·몸통. 높은 Co-occurrence여도 독립 Feature 유지.
+· 'The Torso Extends Backward To Recover Balance.'는 Head Elevation 등 자세 보상 계열에서 재사용되는 표준 Mechanism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="22" customHeight="1">
+      <c r="A162" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B161" s="2" t="inlineStr">
-        <is>
-          <t>Lead Pressure Insufficient  (리드측 압력 부족)   ·   Pressure / Location/Magnitude · Lead·Insufficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="3" t="inlineStr">
-        <is>
-          <t>■ 정의</t>
-        </is>
-      </c>
-      <c r="B162" s="4" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 압력 중심(COP)이 정상보다 충분히 리드측으로 이동하지 못한 현상. 체중 이동 자체보다 리드측 지면반력이 충분히 형성되지 않는 것이 핵심이다.</t>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Head Elevation  (머리 상승)   ·   Head / Position/Height · Rise</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 머리 높이가 정상보다 상승하는 현상. 목만이 아니라 몸 전체의 수직 움직임·자세 변화로 머리가 위로 이동하는 것이 핵심이다. Result Feature 성격이 강하다(In-degree 높음).</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
           <t>■ 원인 추정</t>
         </is>
       </c>
-      <c r="B163" s="4" t="inlineStr">
-        <is>
-          <t>Reverse Pivot (리버스 피벗)
-   ↓
-Pressure Remains On The Trail Side.
-(압력이 트레일측에 남아있다.)
-   ↓
-Lead Pressure Insufficient (리드측 압력 부족)</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="4" t="inlineStr"/>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>Late Pressure Shift (압력 이동 지연)
-   ↓
-Pressure Does Not Reach The Lead Side Before Impact.
-(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
-   ↓
-Lead Pressure Insufficient (리드측 압력 부족)</t>
+          <t>Early Extension (얼리 익스텐션)
+   ↓
+The Head Rises As The Body Stands Up.
+(몸이 일어나면서 머리가 상승한다.)
+   ↓
+Head Elevation (머리 상승)</t>
         </is>
       </c>
     </row>
@@ -2703,12 +2760,12 @@
       <c r="A165" s="4" t="inlineStr"/>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Hanging Back (체중 뒤잔류)
-   ↓
-The Center Of Pressure Stays Behind The Lead Foot.
-(압력 중심이 리드발까지 이동하지 못한다.)
-   ↓
-Lead Pressure Insufficient (리드측 압력 부족)</t>
+          <t>Spine Extension Excessive (척추 과신전)
+   ↓
+The Head Rises As The Body Stands Up.
+(몸이 일어나면서 머리가 상승한다.)
+   ↓
+Head Elevation (머리 상승)</t>
         </is>
       </c>
     </row>
@@ -2716,12 +2773,12 @@
       <c r="A166" s="4" t="inlineStr"/>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
-   ↓
-Body Mass Does Not Continue Moving Toward The Lead Side.
-(몸의 질량이 리드측으로 계속 이동하지 못한다.)
-   ↓
-Lead Pressure Insufficient (리드측 압력 부족)</t>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+The Torso Extends Backward To Recover Balance.
+(균형 회복을 위해 상체가 뒤로 신전한다.)
+   ↓
+Head Elevation (머리 상승)</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2786,12 @@
       <c r="A167" s="4" t="inlineStr"/>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>Lead Hip Internal Rotation Restriction (리드 고관절 내회전 제한)
-   ↓
-The Lead Hip Cannot Accept Rotational Load.
-(리드 고관절이 회전 하중을 받아주지 못한다.)
-   ↓
-Lead Pressure Insufficient (리드측 압력 부족)</t>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+Head Elevation (머리 상승)</t>
         </is>
       </c>
     </row>
@@ -2742,12 +2799,12 @@
       <c r="A168" s="4" t="inlineStr"/>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>Trail Side Push Deficit (트레일측 지면 밀기 부족)
-   ↓
-Insufficient Ground Force Limits Pressure Transfer.
-(지면반력이 부족하여 압력이 리드측으로 전달되지 못한다.)
-   ↓
-Lead Pressure Insufficient (리드측 압력 부족)</t>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+The Lead Side Cannot Become The Primary Rotation Axis.
+(리드측이 주 회전축이 되지 못한다.)
+   ↓
+Head Elevation (머리 상승)</t>
         </is>
       </c>
     </row>
@@ -2759,12 +2816,12 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>Lead Pressure Insufficient (리드측 압력 부족)
-   ↓
-The Body Rotates Around The Trail Side.
-(몸이 트레일측을 중심으로 회전한다.)
-   ↓
-Hanging Back (체중 뒤잔류)</t>
+          <t>Head Elevation (머리 상승)
+   ↓
+The Body Loses Delivery Space.
+(다운스윙 공간이 부족해진다.)
+   ↓
+Handle Raise (핸들 상승)</t>
         </is>
       </c>
     </row>
@@ -2772,14 +2829,12 @@
       <c r="A170" s="4" t="inlineStr"/>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>Lead Pressure Insufficient (리드측 압력 부족)
-   ↓
-The Swing Center Remains Behind The Ball.
-(스윙 중심이 볼 뒤에 남는다.)
-   ↓
-Low Point Variability Increase (최저점 변동 증가)
-   ↓
-Fat Contact (뒤땅)</t>
+          <t>Head Elevation (머리 상승)
+   ↓
+The Swing Axis Shifts Upward.
+(회전축이 위로 이동한다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
         </is>
       </c>
     </row>
@@ -2787,12 +2842,12 @@
       <c r="A171" s="4" t="inlineStr"/>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Lead Pressure Insufficient (리드측 압력 부족)
-   ↓
-The Arms Continue Driving Instead Of Rotating Around The Lead Side.
-(리드측 회전 대신 팔 위주의 전달이 이루어진다.)
-   ↓
-Casting (캐스팅)</t>
+          <t>Head Elevation (머리 상승)
+   ↓
+The Club Approaches From A Steeper Delivery Pattern.
+(클럽이 가파른 전달 패턴으로 접근한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
         </is>
       </c>
     </row>
@@ -2800,6 +2855,571 @@
       <c r="A172" s="4" t="inlineStr"/>
       <c r="B172" s="4" t="inlineStr">
         <is>
+          <t>Head Elevation (머리 상승)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t>· Early Extension (얼리 익스텐션)
+· Spine Extension Excessive (척추 과신전)
+· Handle Raise (핸들 상승)
+· Head Hanging Back (머리 뒤잔류)
+· Hanging Back (체중 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>· Subtype: Spine Dominant / Early Extension / Balance Type 중 어느 경로가 주된지 기록.
+· P6에서는 초기 발생, P7에서 최종 관찰되는 경우가 많음 → 두 구간 체크 대상 (P7 시트 연계).</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t>· Head는 Vertical Axis(Elevation/Drop)와 Horizontal Axis(Hanging Back)로 분리 관리. Elevation은 Early Extension/Spine Extension과 강한 연관.
+· In-degree가 매우 높은 Result Feature — 원인 추론의 관측 지표로 활용.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="22" customHeight="1">
+      <c r="A177" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>Head Drop  (머리 하강)   ·   Head / Position/Height · Drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 머리 높이가 정상보다 과도하게 낮아지는 현상. 정상적 지면반응·측굴에 의한 자연스러운 하강이 아니라 상체가 숙여지며 머리가 낮아지는 것이 핵심이다. Head Elevation과 단순 반대 개념이 아니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>Spine Flexion Excessive (척추 과굴곡)
+   ↓
+The Torso Flexes Excessively And The Head Drops.
+(상체가 과도하게 굴곡되며 머리가 낮아진다.)
+   ↓
+Head Drop (머리 하강)</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr"/>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>Trail Side Bend Excessive (트레일측 측굴 과다)
+   ↓
+Excessive Trail Side Bend Lowers The Head.
+(과도한 트레일측 측굴로 머리가 낮아진다.)
+   ↓
+Head Drop (머리 하강)</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr"/>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive (리드측 압력 과다)
+   ↓
+Pressure On The Lead Side Becomes Excessive.
+(리드측 압력이 과도해진다.)
+   ↓
+Head Drop (머리 하강)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>Head Drop (머리 하강)
+   ↓
+The Body Moves Toward The Ball And Loses Space.
+(몸이 볼 방향으로 이동하며 공간을 잃는다.)
+   ↓
+Handle Too Low (핸들 낮음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="4" t="inlineStr"/>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>Head Drop (머리 하강)
+   ↓
+The Club Approaches From Inside.
+(클럽이 안쪽 경로로 접근한다.)
+   ↓
+Deep Hands (손 깊음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="4" t="inlineStr"/>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>Head Drop (머리 하강)
+   ↓
+The Club Bottoms Out Behind The Ball.
+(클럽 최저점이 볼 뒤에서 형성된다.)
+   ↓
+Fat Contact (뒤땅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="4" t="inlineStr"/>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>Head Drop (머리 하강)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Closed (클럽페이스 클로즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>· Spine Flexion Excessive (척추 과굴곡)
+· Trail Side Bend Excessive (트레일측 측굴 과다)
+· Deep Hands (손 깊음)
+· Handle Too Low (핸들 낮음)
+· Hanging Back (체중 뒤잔류)
+· Club Face Closed (클럽페이스 클로즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>· Head Elevation과 단순 ± 관계가 아님 — 원인·결과 Chain이 완전히 다름.
+· Subtype: Side Bend Type / Flexion Type / Handle Type 구분.
+· 명명: 다운스윙의 약간의 머리 하강은 정상일 수 있으므로 'Excessive Head Drop' 명명 검토.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>· Head Vertical Motion은 Elevation과 Drop 두 방향이며 서로 다른 Chain을 가진 독립 Observation.
+· Head Drop → Spine Flexion / Side Bend / 손 위치 변화와 강한 연관 (Elevation의 Spine Extension 계열과 대비).</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="22" customHeight="1">
+      <c r="A190" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Head Hanging Back  (머리 뒤잔류)   ·   Head / Position/Location · Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 머리 위치가 정상보다 후방(트레일측)에 남아 목표 방향으로 이동하지 못하는 현상. 체중 패턴(Hanging Back)과는 별개의 머리 위치 Feature이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+The Head Remains On The Trail Side.
+(머리가 트레일측에 남는다.)
+   ↓
+Head Hanging Back (머리 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="4" t="inlineStr"/>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>Late Pressure Shift (압력 이동 지연)
+   ↓
+The Head Remains On The Trail Side.
+(머리가 트레일측에 남는다.)
+   ↓
+Head Hanging Back (머리 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="4" t="inlineStr"/>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+Pressure Remains On The Trail Side.
+(압력이 트레일측에 남아있다.)
+   ↓
+Head Hanging Back (머리 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr"/>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Insufficient (골반 회전 부족)
+   ↓
+Pelvis Rotation Does Not Complete Through Impact.
+(골반 회전이 임팩트까지 완성되지 않는다.)
+   ↓
+Head Hanging Back (머리 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="4" t="inlineStr"/>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Stall (골반 회전 정지)
+   ↓
+Pelvis Rotation Decelerates Before Impact.
+(임팩트 전에 골반 회전이 감속한다.)
+   ↓
+Head Hanging Back (머리 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t>Head Hanging Back (머리 뒤잔류)
+   ↓
+The Swing Center Remains Behind The Ball.
+(스윙 중심이 볼 뒤에 남는다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr"/>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>Head Hanging Back (머리 뒤잔류)
+   ↓
+Pressure Remains On The Trail Side.
+(압력이 트레일측에 남아있다.)
+   ↓
+Hanging Back (체중 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="4" t="inlineStr"/>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>Head Hanging Back (머리 뒤잔류)
+   ↓
+The Club Bottoms Out Behind The Ball.
+(클럽 최저점이 볼 뒤에서 형성된다.)
+   ↓
+Fat Contact (뒤땅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="4" t="inlineStr"/>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>Head Hanging Back (머리 뒤잔류)
+   ↓
+The Club Face Cannot Square In Time.
+(클럽페이스가 제시간에 스퀘어되지 못한다.)
+   ↓
+Club Face Open (클럽페이스 오픈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t>· Hanging Back (체중 뒤잔류)
+· Lead Pressure Insufficient (리드측 압력 부족)
+· Late Pressure Shift (압력 이동 지연)
+· Early Extension (얼리 익스텐션)
+· Head Elevation (머리 상승)
+· Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>· Head Hanging Back(머리 위치) ≠ Hanging Back(체중 패턴) — 독립 Feature 유지 근거 재확인.
+· 체중은 이동했지만 머리만 뒤에 남는 Head-only Type이 실제로 얼마나 존재하는지 확인.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>· Head는 Vertical(Elevation/Drop)과 Horizontal(Hanging Back)로 분리. Hanging Back은 수평축(Trail 방향).
+· 이후 Head Moving Forward를 추가해도 동일 체계(수직/수평)로 관리 가능.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="22" customHeight="1">
+      <c r="A205" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient  (리드측 압력 부족)   ·   Pressure / Location/Magnitude · Lead·Insufficient</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 압력 중심(COP)이 정상보다 충분히 리드측으로 이동하지 못한 현상. 체중 이동 자체보다 리드측 지면반력이 충분히 형성되지 않는 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>Reverse Pivot (리버스 피벗)
+   ↓
+Pressure Remains On The Trail Side.
+(압력이 트레일측에 남아있다.)
+   ↓
+Lead Pressure Insufficient (리드측 압력 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="4" t="inlineStr"/>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>Late Pressure Shift (압력 이동 지연)
+   ↓
+Pressure Does Not Reach The Lead Side Before Impact.
+(임팩트 전까지 압력이 리드측에 도달하지 못한다.)
+   ↓
+Lead Pressure Insufficient (리드측 압력 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="4" t="inlineStr"/>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t>Hanging Back (체중 뒤잔류)
+   ↓
+The Center Of Pressure Stays Behind The Lead Foot.
+(압력 중심이 리드발까지 이동하지 못한다.)
+   ↓
+Lead Pressure Insufficient (리드측 압력 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="4" t="inlineStr"/>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient (흉곽 회전 부족)
+   ↓
+Body Mass Does Not Continue Moving Toward The Lead Side.
+(몸의 질량이 리드측으로 계속 이동하지 못한다.)
+   ↓
+Lead Pressure Insufficient (리드측 압력 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr"/>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>Lead Hip Internal Rotation Restriction (리드 고관절 내회전 제한)
+   ↓
+The Lead Hip Cannot Accept Rotational Load.
+(리드 고관절이 회전 하중을 받아주지 못한다.)
+   ↓
+Lead Pressure Insufficient (리드측 압력 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="inlineStr"/>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>Trail Side Push Deficit (트레일측 지면 밀기 부족)
+   ↓
+Insufficient Ground Force Limits Pressure Transfer.
+(지면반력이 부족하여 압력이 리드측으로 전달되지 못한다.)
+   ↓
+Lead Pressure Insufficient (리드측 압력 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+The Body Rotates Around The Trail Side.
+(몸이 트레일측을 중심으로 회전한다.)
+   ↓
+Hanging Back (체중 뒤잔류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="4" t="inlineStr"/>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+The Swing Center Remains Behind The Ball.
+(스윙 중심이 볼 뒤에 남는다.)
+   ↓
+Low Point Variability Increase (최저점 변동 증가)
+   ↓
+Fat Contact (뒤땅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr"/>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+The Arms Continue Driving Instead Of Rotating Around The Lead Side.
+(리드측 회전 대신 팔 위주의 전달이 이루어진다.)
+   ↓
+Casting (캐스팅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="4" t="inlineStr"/>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
           <t>Lead Pressure Insufficient (리드측 압력 부족)
    ↓
 The Trail Side Continues Supporting Rotation.
@@ -2809,9 +3429,9 @@
         </is>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" s="4" t="inlineStr"/>
-      <c r="B173" s="4" t="inlineStr">
+    <row r="217">
+      <c r="A217" s="4" t="inlineStr"/>
+      <c r="B217" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Insufficient (리드측 압력 부족)
    ↓
@@ -2824,9 +3444,9 @@
         </is>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="4" t="inlineStr"/>
-      <c r="B174" s="4" t="inlineStr">
+    <row r="218">
+      <c r="A218" s="4" t="inlineStr"/>
+      <c r="B218" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Insufficient (리드측 압력 부족)
    ↓
@@ -2837,30 +3457,30 @@
         </is>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="3" t="inlineStr">
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
         <is>
           <t>■ Strong Co-occurrence</t>
         </is>
       </c>
-      <c r="B175" s="4" t="inlineStr">
-        <is>
-          <t>★★★★★ Late Pressure Shift (압력 이동 지연)
-★★★★★ Hanging Back (체중 뒤잔류)
-★★★★★ Spin-out (스핀아웃)
-★★★★☆ Casting (캐스팅)
-★★★★☆ Pelvis Rotation Insufficient (골반 회전 부족)
-★★★★☆ Thorax Rotation Insufficient (흉곽 회전 부족)</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="3" t="inlineStr">
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t>· Late Pressure Shift (압력 이동 지연)
+· Hanging Back (체중 뒤잔류)
+· Spin-out (스핀아웃)
+· Casting (캐스팅)
+· Pelvis Rotation Insufficient (골반 회전 부족)
+· Thorax Rotation Insufficient (흉곽 회전 부족)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
         <is>
           <t>■ 추가 검증 포인트</t>
         </is>
       </c>
-      <c r="B176" s="4" t="inlineStr">
+      <c r="B220" s="4" t="inlineStr">
         <is>
           <t>① Lead Pressure Insufficient(COP)와 Hanging Back(COM)은 서로 다른 Observation — 직접 인과인지 Common Cause인지 검증.
 ② Pelvis Slide Excessive가 항상 리드측 압력 부족으로 이어지지는 않음 (슬라이드 방식/회전 동반 여부에 따라 다름).
@@ -2868,13 +3488,13 @@
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="3" t="inlineStr">
+    <row r="221">
+      <c r="A221" s="3" t="inlineStr">
         <is>
           <t>■ 사고확장</t>
         </is>
       </c>
-      <c r="B177" s="4" t="inlineStr">
+      <c r="B221" s="4" t="inlineStr">
         <is>
           <t>① 본질은 단순 압력 부족이 아니라 '리드측을 회전축으로 사용하지 못하는 상태'일 가능성 (압력 &lt; 회전축 형성 실패).
 ② 발생 시 팔이 클럽을 전달하는 비율 증가 → Body Driven → Arm Driven 전환의 중간 과정.
@@ -2882,37 +3502,37 @@
         </is>
       </c>
     </row>
-    <row r="179" ht="22" customHeight="1">
-      <c r="A179" s="1" t="inlineStr">
+    <row r="223" ht="22" customHeight="1">
+      <c r="A223" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B223" s="2" t="inlineStr">
         <is>
           <t>Lead Pressure Excessive  (리드측 압력 과다)   ·   Pressure / Location/Magnitude · Lead·Excessive</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="3" t="inlineStr">
+    <row r="224">
+      <c r="A224" s="3" t="inlineStr">
         <is>
           <t>■ 정의</t>
         </is>
       </c>
-      <c r="B180" s="4" t="inlineStr">
+      <c r="B224" s="4" t="inlineStr">
         <is>
           <t>다운스윙 중반(P6)에서 압력 중심(COP)이 정상보다 과도하게 리드측에 집중되는 현상. 단순히 왼발 체중이 많은 것이 아니라 압력 이동의 양 또는 속도가 과도하여 정상적인 회전·클럽 전달에 영향을 주는 것이 핵심이다.</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="3" t="inlineStr">
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr">
         <is>
           <t>■ 원인 추정</t>
         </is>
       </c>
-      <c r="B181" s="4" t="inlineStr">
+      <c r="B225" s="4" t="inlineStr">
         <is>
           <t>Early Pressure Shift (조기 압력 이동)
    ↓
@@ -2923,9 +3543,9 @@
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="4" t="inlineStr"/>
-      <c r="B182" s="4" t="inlineStr">
+    <row r="226">
+      <c r="A226" s="4" t="inlineStr"/>
+      <c r="B226" s="4" t="inlineStr">
         <is>
           <t>Pelvis Slide Excessive (과도한 골반 슬라이드)
    ↓
@@ -2936,9 +3556,9 @@
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="4" t="inlineStr"/>
-      <c r="B183" s="4" t="inlineStr">
+    <row r="227">
+      <c r="A227" s="4" t="inlineStr"/>
+      <c r="B227" s="4" t="inlineStr">
         <is>
           <t>Trail Side Push Excessive (트레일측 과도한 지면 밀기)
    ↓
@@ -2949,9 +3569,9 @@
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="4" t="inlineStr"/>
-      <c r="B184" s="4" t="inlineStr">
+    <row r="228">
+      <c r="A228" s="4" t="inlineStr"/>
+      <c r="B228" s="4" t="inlineStr">
         <is>
           <t>Insufficient Trail Side Pressure During Backswing (백스윙 트레일측 압력 부족)
    ↓
@@ -2965,9 +3585,9 @@
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="4" t="inlineStr"/>
-      <c r="B185" s="4" t="inlineStr">
+    <row r="229">
+      <c r="A229" s="4" t="inlineStr"/>
+      <c r="B229" s="4" t="inlineStr">
         <is>
           <t>Lead Hip Internal Rotation Restriction / Lead Glute·Adductor Underactivation (리드 고관절 내회전 제한 / 리드 둔근·내전근 활성 부족)
    ↓
@@ -2978,13 +3598,13 @@
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="3" t="inlineStr">
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
         <is>
           <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
-      <c r="B186" s="4" t="inlineStr">
+      <c r="B230" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Excessive (리드측 압력 과다)
    ↓
@@ -2995,9 +3615,9 @@
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="4" t="inlineStr"/>
-      <c r="B187" s="4" t="inlineStr">
+    <row r="231">
+      <c r="A231" s="4" t="inlineStr"/>
+      <c r="B231" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Excessive (리드측 압력 과다)
    ↓
@@ -3008,9 +3628,9 @@
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="4" t="inlineStr"/>
-      <c r="B188" s="4" t="inlineStr">
+    <row r="232">
+      <c r="A232" s="4" t="inlineStr"/>
+      <c r="B232" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Excessive (리드측 압력 과다)
    ↓
@@ -3021,9 +3641,9 @@
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="4" t="inlineStr"/>
-      <c r="B189" s="4" t="inlineStr">
+    <row r="233">
+      <c r="A233" s="4" t="inlineStr"/>
+      <c r="B233" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Excessive (리드측 압력 과다)
    ↓
@@ -3034,9 +3654,9 @@
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="4" t="inlineStr"/>
-      <c r="B190" s="4" t="inlineStr">
+    <row r="234">
+      <c r="A234" s="4" t="inlineStr"/>
+      <c r="B234" s="4" t="inlineStr">
         <is>
           <t>Lead Pressure Excessive (리드측 압력 과다)
    ↓
@@ -3050,81 +3670,81 @@
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="3" t="inlineStr">
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
         <is>
           <t>■ Strong Co-occurrence</t>
         </is>
       </c>
-      <c r="B191" s="4" t="inlineStr">
-        <is>
-          <t>★★★★★ Early Pressure Shift (조기 압력 이동)
-★★★★★ Pelvis Slide Excessive (과도한 골반 슬라이드)
-★★★★★ Casting (캐스팅)
-★★★★☆ Late Arm (팔 하강 지연)
-★★★★☆ Pelvis Open Early (골반 조기 오픈)
-★★★★☆ Thorax Open Early (흉곽 조기 오픈)
-★★★★☆ Early Extension (얼리 익스텐션)</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="3" t="inlineStr">
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>· Early Pressure Shift (조기 압력 이동)
+· Pelvis Slide Excessive (과도한 골반 슬라이드)
+· Casting (캐스팅)
+· Late Arm (팔 하강 지연)
+· Pelvis Open Early (골반 조기 오픈)
+· Thorax Open Early (흉곽 조기 오픈)
+· Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
         <is>
           <t>■ 추가 검증 포인트</t>
         </is>
       </c>
-      <c r="B192" s="4" t="inlineStr">
+      <c r="B236" s="4" t="inlineStr">
         <is>
           <t>① Lead Pressure Insufficient와 Lead Pressure Excessive는 둘 다 Casting으로 이어질 수 있으나 메커니즘이 완전히 다르다: Insufficient=공에 도달하려 캐스팅 / Excessive=몸이 앞서가 타이밍 맞추려 캐스팅. 같은 결과·다른 원인 구분이 DOH의 핵심 가치.
 ② Cross-over Top Pattern(P4)은 Lead Pressure Excessive + Thoracic Hyperextension 복합에서 자주 관찰 → 독립 Feature보다 Composite Observation 후보로 검증.</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="3" t="inlineStr">
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
         <is>
           <t>■ 사고확장</t>
         </is>
       </c>
-      <c r="B193" s="4" t="inlineStr">
+      <c r="B237" s="4" t="inlineStr">
         <is>
           <t>· 'The Lead Knee And Hip Drift Excessively Toward The Target.'는 무릎·고관절·압력 Feature를 잇는 중간 Mechanism으로 저장 가치가 높아 Dictionary에 등록함 (향후 재사용).
 · Cross-over Top Pattern은 P4 Composite Observation 후보로 별도 기록 (Feature_Dictionary candidate).</t>
         </is>
       </c>
     </row>
-    <row r="195" ht="22" customHeight="1">
-      <c r="A195" s="1" t="inlineStr">
+    <row r="239" ht="22" customHeight="1">
+      <c r="A239" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B239" s="2" t="inlineStr">
         <is>
           <t>Incomplete Pressure Transfer  (압력 이동 미완성)   ·   Pressure / Timing · Late</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="3" t="inlineStr">
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
         <is>
           <t>■ 정의</t>
         </is>
       </c>
-      <c r="B196" s="4" t="inlineStr">
+      <c r="B240" s="4" t="inlineStr">
         <is>
           <t>다운스윙(P4~P7) 과정에서 압력이 정상적으로 리드측까지 전달되지 못한 현상. 이동 속도(Timing)가 아니라 임팩트(P7)까지 충분한 리드측 압력이 형성되지 않는 것이 핵심이며, 이동이 늦거나·부족하거나·중간에 멈추는 경우를 모두 포함한다.</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="3" t="inlineStr">
+    <row r="241">
+      <c r="A241" s="3" t="inlineStr">
         <is>
           <t>■ 원인 추정</t>
         </is>
       </c>
-      <c r="B197" s="4" t="inlineStr">
+      <c r="B241" s="4" t="inlineStr">
         <is>
           <t>Reverse Pivot (리버스 피벗)
    ↓
@@ -3135,9 +3755,9 @@
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="4" t="inlineStr"/>
-      <c r="B198" s="4" t="inlineStr">
+    <row r="242">
+      <c r="A242" s="4" t="inlineStr"/>
+      <c r="B242" s="4" t="inlineStr">
         <is>
           <t>Insufficient Trail Side Loading During Backswing (백스윙 트레일측 압력 형성 부족)
    ↓
@@ -3148,9 +3768,9 @@
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="4" t="inlineStr"/>
-      <c r="B199" s="4" t="inlineStr">
+    <row r="243">
+      <c r="A243" s="4" t="inlineStr"/>
+      <c r="B243" s="4" t="inlineStr">
         <is>
           <t>Lead Hip Internal Rotation Restriction (리드 고관절 내회전 제한)
    ↓
@@ -3161,9 +3781,9 @@
         </is>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="4" t="inlineStr"/>
-      <c r="B200" s="4" t="inlineStr">
+    <row r="244">
+      <c r="A244" s="4" t="inlineStr"/>
+      <c r="B244" s="4" t="inlineStr">
         <is>
           <t>Lead Glute·Adductor Underactivation (리드 둔근·내전근 활성 부족)
    ↓
@@ -3174,9 +3794,9 @@
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="4" t="inlineStr"/>
-      <c r="B201" s="4" t="inlineStr">
+    <row r="245">
+      <c r="A245" s="4" t="inlineStr"/>
+      <c r="B245" s="4" t="inlineStr">
         <is>
           <t>Hanging Back (체중 뒤잔류)
    ↓
@@ -3187,13 +3807,13 @@
         </is>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="3" t="inlineStr">
+    <row r="246">
+      <c r="A246" s="3" t="inlineStr">
         <is>
           <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
-      <c r="B202" s="4" t="inlineStr">
+      <c r="B246" s="4" t="inlineStr">
         <is>
           <t>Incomplete Pressure Transfer (압력 이동 미완성)
    ↓
@@ -3204,9 +3824,9 @@
         </is>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" s="4" t="inlineStr"/>
-      <c r="B203" s="4" t="inlineStr">
+    <row r="247">
+      <c r="A247" s="4" t="inlineStr"/>
+      <c r="B247" s="4" t="inlineStr">
         <is>
           <t>Incomplete Pressure Transfer (압력 이동 미완성)
    ↓
@@ -3219,9 +3839,9 @@
         </is>
       </c>
     </row>
-    <row r="204">
-      <c r="A204" s="4" t="inlineStr"/>
-      <c r="B204" s="4" t="inlineStr">
+    <row r="248">
+      <c r="A248" s="4" t="inlineStr"/>
+      <c r="B248" s="4" t="inlineStr">
         <is>
           <t>Incomplete Pressure Transfer (압력 이동 미완성)
    ↓
@@ -3232,9 +3852,9 @@
         </is>
       </c>
     </row>
-    <row r="205">
-      <c r="A205" s="4" t="inlineStr"/>
-      <c r="B205" s="4" t="inlineStr">
+    <row r="249">
+      <c r="A249" s="4" t="inlineStr"/>
+      <c r="B249" s="4" t="inlineStr">
         <is>
           <t>Incomplete Pressure Transfer (압력 이동 미완성)
    ↓
@@ -3245,9 +3865,9 @@
         </is>
       </c>
     </row>
-    <row r="206">
-      <c r="A206" s="4" t="inlineStr"/>
-      <c r="B206" s="4" t="inlineStr">
+    <row r="250">
+      <c r="A250" s="4" t="inlineStr"/>
+      <c r="B250" s="4" t="inlineStr">
         <is>
           <t>Incomplete Pressure Transfer (압력 이동 미완성)
    ↓
@@ -3258,43 +3878,43 @@
         </is>
       </c>
     </row>
-    <row r="207">
-      <c r="A207" s="3" t="inlineStr">
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
         <is>
           <t>■ Strong Co-occurrence</t>
         </is>
       </c>
-      <c r="B207" s="4" t="inlineStr">
-        <is>
-          <t>★★★★★ Lead Pressure Insufficient (리드측 압력 부족)
-★★★★★ Hanging Back (체중 뒤잔류)
-★★★★★ Casting (캐스팅)
-★★★★☆ Pelvis Rotation Insufficient (골반 회전 부족)
-★★★★☆ Thorax Rotation Insufficient (흉곽 회전 부족)
-★★★★☆ Spin-out (스핀아웃)</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="3" t="inlineStr">
+      <c r="B251" s="4" t="inlineStr">
+        <is>
+          <t>· Lead Pressure Insufficient (리드측 압력 부족)
+· Hanging Back (체중 뒤잔류)
+· Casting (캐스팅)
+· Pelvis Rotation Insufficient (골반 회전 부족)
+· Thorax Rotation Insufficient (흉곽 회전 부족)
+· Spin-out (스핀아웃)</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
         <is>
           <t>■ 추가 검증 포인트</t>
         </is>
       </c>
-      <c r="B208" s="4" t="inlineStr">
+      <c r="B252" s="4" t="inlineStr">
         <is>
           <t>① Incomplete Pressure Transfer와 Lead Pressure Insufficient를 독립 Feature로 유지할지, 하나로 통합할지 검증.
 ② 압력 이동이 '부족한 경우'와 '완료됐지만 Timing만 늦은 경우'를 구분할 필요가 있는지 검증.</t>
         </is>
       </c>
     </row>
-    <row r="209">
-      <c r="A209" s="3" t="inlineStr">
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
         <is>
           <t>■ 사고확장</t>
         </is>
       </c>
-      <c r="B209" s="4" t="inlineStr">
+      <c r="B253" s="4" t="inlineStr">
         <is>
           <t>① 압력 이동 실패의 본질은 '압력'보다 '회전축 형성 실패'일 가능성.
 ② P6에서 관찰되지만 실제 원인은 대부분 P1~P4에서 이미 결정될 가능성.
@@ -3302,37 +3922,37 @@
         </is>
       </c>
     </row>
-    <row r="211" ht="22" customHeight="1">
-      <c r="A211" s="1" t="inlineStr">
+    <row r="255" ht="22" customHeight="1">
+      <c r="A255" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B211" s="2" t="inlineStr">
+      <c r="B255" s="2" t="inlineStr">
         <is>
           <t>High Hands  (손 높음)   ·   Hands / Position/Height · High (Relative)</t>
         </is>
       </c>
     </row>
-    <row r="212">
-      <c r="A212" s="3" t="inlineStr">
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
         <is>
           <t>■ 정의</t>
         </is>
       </c>
-      <c r="B212" s="4" t="inlineStr">
+      <c r="B256" s="4" t="inlineStr">
         <is>
           <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 높은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 충분히 하강하지 못한 상대 위치가 핵심이다.</t>
         </is>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" s="3" t="inlineStr">
+    <row r="257">
+      <c r="A257" s="3" t="inlineStr">
         <is>
           <t>■ 원인 추정</t>
         </is>
       </c>
-      <c r="B213" s="4" t="inlineStr">
+      <c r="B257" s="4" t="inlineStr">
         <is>
           <t>Arm Depth Excessive (P4, 백스윙 손 과도한 깊이)
    ↓
@@ -3349,9 +3969,9 @@
         </is>
       </c>
     </row>
-    <row r="214">
-      <c r="A214" s="4" t="inlineStr"/>
-      <c r="B214" s="4" t="inlineStr">
+    <row r="258">
+      <c r="A258" s="4" t="inlineStr"/>
+      <c r="B258" s="4" t="inlineStr">
         <is>
           <t>Arm Drop Insufficient (팔 하강 부족)
    ↓
@@ -3362,9 +3982,9 @@
         </is>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="4" t="inlineStr"/>
-      <c r="B215" s="4" t="inlineStr">
+    <row r="259">
+      <c r="A259" s="4" t="inlineStr"/>
+      <c r="B259" s="4" t="inlineStr">
         <is>
           <t>Early Extension (얼리 익스텐션)
    ↓
@@ -3375,13 +3995,13 @@
         </is>
       </c>
     </row>
-    <row r="216">
-      <c r="A216" s="3" t="inlineStr">
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
         <is>
           <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
-      <c r="B216" s="4" t="inlineStr">
+      <c r="B260" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -3392,9 +4012,9 @@
         </is>
       </c>
     </row>
-    <row r="217">
-      <c r="A217" s="4" t="inlineStr"/>
-      <c r="B217" s="4" t="inlineStr">
+    <row r="261">
+      <c r="A261" s="4" t="inlineStr"/>
+      <c r="B261" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -3405,9 +4025,9 @@
         </is>
       </c>
     </row>
-    <row r="218">
-      <c r="A218" s="4" t="inlineStr"/>
-      <c r="B218" s="4" t="inlineStr">
+    <row r="262">
+      <c r="A262" s="4" t="inlineStr"/>
+      <c r="B262" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -3420,9 +4040,9 @@
         </is>
       </c>
     </row>
-    <row r="219">
-      <c r="A219" s="4" t="inlineStr"/>
-      <c r="B219" s="4" t="inlineStr">
+    <row r="263">
+      <c r="A263" s="4" t="inlineStr"/>
+      <c r="B263" s="4" t="inlineStr">
         <is>
           <t>High Hands (손 높음)
    ↓
@@ -3433,13 +4053,13 @@
         </is>
       </c>
     </row>
-    <row r="220">
-      <c r="A220" s="3" t="inlineStr">
+    <row r="264">
+      <c r="A264" s="3" t="inlineStr">
         <is>
           <t>■ Strong Co-occurrence</t>
         </is>
       </c>
-      <c r="B220" s="4" t="inlineStr">
+      <c r="B264" s="4" t="inlineStr">
         <is>
           <t>· Steep Shaft (가파른 샤프트)
 · Handle Raise (핸들 상승)
@@ -3448,267 +4068,267 @@
         </is>
       </c>
     </row>
-    <row r="221">
-      <c r="A221" s="3" t="inlineStr">
+    <row r="265">
+      <c r="A265" s="3" t="inlineStr">
         <is>
           <t>■ 추가 검증 포인트</t>
         </is>
       </c>
-      <c r="B221" s="4" t="inlineStr">
+      <c r="B265" s="4" t="inlineStr">
         <is>
           <t>· High Hands가 '손이 높아서'인지 '몸의 회전에 비해 손이 늦게 내려와서'인지 레슨 데이터로 구분 필요 (후자 가능성 높음).
 · High Hands → Steep Shaft는 흔한 조합이나, 높은 손에서도 샤프트를 눕혀 전달하는 예외 골퍼 존재 여부 확인.</t>
         </is>
       </c>
     </row>
-    <row r="222">
-      <c r="A222" s="3" t="inlineStr">
+    <row r="266">
+      <c r="A266" s="3" t="inlineStr">
         <is>
           <t>■ 사고확장</t>
         </is>
       </c>
-      <c r="B222" s="4" t="inlineStr">
+      <c r="B266" s="4" t="inlineStr">
         <is>
           <t>· P6 손 위치 Feature는 모두 상대 위치(Relative Position): '이 시점의 다운스윙 진행에서 정상이라면 손이 어디 있어야 하는가' 기준. High/Low/Deep/Shallow 전부 동일 철학.
 · High Hands는 P4→Transition→P6를 잇는 Cross-Phase Chain의 대표 사례. P7 Steep Shaft/Outside Delivery로 이어진다.</t>
         </is>
       </c>
     </row>
-    <row r="224" ht="22" customHeight="1">
-      <c r="A224" s="1" t="inlineStr">
+    <row r="268" ht="22" customHeight="1">
+      <c r="A268" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B224" s="2" t="inlineStr">
+      <c r="B268" s="2" t="inlineStr">
         <is>
           <t>Low Hands  (손 낮음)   ·   Hands / Position/Height · Low (Relative)</t>
         </is>
       </c>
     </row>
-    <row r="225">
-      <c r="A225" s="3" t="inlineStr">
+    <row r="269">
+      <c r="A269" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B225" s="4" t="inlineStr">
+      <c r="B269" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="227" ht="22" customHeight="1">
-      <c r="A227" s="1" t="inlineStr">
+    <row r="271" ht="22" customHeight="1">
+      <c r="A271" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B227" s="2" t="inlineStr">
+      <c r="B271" s="2" t="inlineStr">
         <is>
           <t>Deep Hands  (손 깊음)   ·   Hands / Position/Depth · Deep</t>
         </is>
       </c>
     </row>
-    <row r="228">
-      <c r="A228" s="3" t="inlineStr">
+    <row r="272">
+      <c r="A272" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B228" s="4" t="inlineStr">
+      <c r="B272" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="230" ht="22" customHeight="1">
-      <c r="A230" s="1" t="inlineStr">
+    <row r="274" ht="22" customHeight="1">
+      <c r="A274" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B230" s="2" t="inlineStr">
+      <c r="B274" s="2" t="inlineStr">
         <is>
           <t>Forward Hands  (손 전방)   ·   Hands / Position/Direction · Forward</t>
         </is>
       </c>
     </row>
-    <row r="231">
-      <c r="A231" s="3" t="inlineStr">
+    <row r="275">
+      <c r="A275" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B231" s="4" t="inlineStr">
+      <c r="B275" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="233" ht="22" customHeight="1">
-      <c r="A233" s="1" t="inlineStr">
+    <row r="277" ht="22" customHeight="1">
+      <c r="A277" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B233" s="2" t="inlineStr">
+      <c r="B277" s="2" t="inlineStr">
         <is>
           <t>Hands Too Far From Body  (손이 몸에서 멀어짐)   ·   Hands / Relationship · Far</t>
         </is>
       </c>
     </row>
-    <row r="234">
-      <c r="A234" s="3" t="inlineStr">
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B234" s="4" t="inlineStr">
+      <c r="B278" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="236" ht="22" customHeight="1">
-      <c r="A236" s="1" t="inlineStr">
+    <row r="280" ht="22" customHeight="1">
+      <c r="A280" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B236" s="2" t="inlineStr">
+      <c r="B280" s="2" t="inlineStr">
         <is>
           <t>Hands Too Close To Body  (손이 몸에 가까움)   ·   Hands / Relationship · Close</t>
         </is>
       </c>
     </row>
-    <row r="237">
-      <c r="A237" s="3" t="inlineStr">
+    <row r="281">
+      <c r="A281" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B237" s="4" t="inlineStr">
+      <c r="B281" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="239" ht="22" customHeight="1">
-      <c r="A239" s="1" t="inlineStr">
+    <row r="283" ht="22" customHeight="1">
+      <c r="A283" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B239" s="2" t="inlineStr">
+      <c r="B283" s="2" t="inlineStr">
         <is>
           <t>Late Arm  (팔 하강 지연)   ·   Arm / Timing · Late</t>
         </is>
       </c>
     </row>
-    <row r="240">
-      <c r="A240" s="3" t="inlineStr">
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B240" s="4" t="inlineStr">
+      <c r="B284" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="242" ht="22" customHeight="1">
-      <c r="A242" s="1" t="inlineStr">
+    <row r="286" ht="22" customHeight="1">
+      <c r="A286" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B242" s="2" t="inlineStr">
+      <c r="B286" s="2" t="inlineStr">
         <is>
           <t>Trail Elbow Behind Body  (트레일 팔꿈치 뒤처짐)   ·   Trail Elbow / Location · Trail</t>
         </is>
       </c>
     </row>
-    <row r="243">
-      <c r="A243" s="3" t="inlineStr">
+    <row r="287">
+      <c r="A287" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B243" s="4" t="inlineStr">
+      <c r="B287" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="245" ht="22" customHeight="1">
-      <c r="A245" s="1" t="inlineStr">
+    <row r="289" ht="22" customHeight="1">
+      <c r="A289" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B245" s="2" t="inlineStr">
+      <c r="B289" s="2" t="inlineStr">
         <is>
           <t>Steep Shaft  (가파른 샤프트)   ·   Shaft / Angle/Plane · Steep</t>
         </is>
       </c>
     </row>
-    <row r="246">
-      <c r="A246" s="3" t="inlineStr">
+    <row r="290">
+      <c r="A290" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B246" s="4" t="inlineStr">
+      <c r="B290" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="248" ht="22" customHeight="1">
-      <c r="A248" s="1" t="inlineStr">
+    <row r="292" ht="22" customHeight="1">
+      <c r="A292" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B248" s="2" t="inlineStr">
+      <c r="B292" s="2" t="inlineStr">
         <is>
           <t>Shallow Shaft  (눕는 샤프트)   ·   Shaft / Angle/Plane · Shallow</t>
         </is>
       </c>
     </row>
-    <row r="249">
-      <c r="A249" s="3" t="inlineStr">
+    <row r="293">
+      <c r="A293" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B249" s="4" t="inlineStr">
+      <c r="B293" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
       </c>
     </row>
-    <row r="251" ht="22" customHeight="1">
-      <c r="A251" s="1" t="inlineStr">
+    <row r="295" ht="22" customHeight="1">
+      <c r="A295" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B251" s="2" t="inlineStr">
+      <c r="B295" s="2" t="inlineStr">
         <is>
           <t>Casting  (캐스팅)   ·   Club / Release · Cast</t>
         </is>
       </c>
     </row>
-    <row r="252">
-      <c r="A252" s="3" t="inlineStr">
+    <row r="296">
+      <c r="A296" s="3" t="inlineStr">
         <is>
           <t>(상태)</t>
         </is>
       </c>
-      <c r="B252" s="4" t="inlineStr">
+      <c r="B296" s="4" t="inlineStr">
         <is>
           <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
         </is>
@@ -3725,7 +4345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5101,105 +5721,138 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
+          <t>The Club Approaches From Inside.</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>클럽이 안쪽 경로로 접근한다.</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Inside Delivery</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>head_drop
+shallow_shaft</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. M-CLB-02(Outside)의 대응 링크.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
           <t>The Club Approaches From Outside.</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>클럽이 바깥쪽 경로로 접근한다.</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>Over The Top
 Outside Delivery
 Out-To-In Path</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>outside_delivery</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>The Club Bottoms Out Behind The Ball.</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>클럽 최저점이 볼 뒤에서 형성된다.</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Low Point Behind Ball
 Bottoms Out Early</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>fat_contact
 head_drop
 head_hanging_back</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>The Club Face Cannot Square In Time.</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>클럽페이스가 제시간에 스퀘어되지 못한다.</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>Face Stays Open
 Face Cannot Rotate In Time</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>club_face_open</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>The Club Is Released Early To Reach The Ball.</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>공에 도달하기 위해 클럽을 조기에 푼다.</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>Casting
 Early Release
@@ -5207,250 +5860,222 @@
 Hand Dominance Release</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>The Clubhead Overtakes The Hands Early.</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>클럽헤드가 손보다 먼저 앞선다.</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Flip
 Clubhead Passes Hands Early
 Scoop</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>flip_release</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Reduced Arm Space Promotes Early Club Release.</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>팔 공간 부족으로 클럽을 조기에 풀게 된다.</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>No Space Forces Casting
 Tight Space Causes Early Release</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>casting
 early_extension</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>The Body Loses Delivery Space.</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>다운스윙 공간이 부족해진다.</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>No Room To Deliver
 Space Collapses</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>early_extension
 high_hands</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="10" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>The Body Moves Toward The Ball And Loses Space.</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>몸이 볼 방향으로 이동하며 공간을 잃는다.</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>Body Drifts To The Ball
 Toward-Ball Movement</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="E52" s="4" t="inlineStr">
         <is>
           <t>early_extension
 high_hands</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+      <c r="F52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>The Body Reaches The Lead Side Before The Arms.</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>몸이 팔보다 먼저 리드측에 도달한다.</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>Body Ahead Of Arms Into Impact
 Body Gets Left First</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early
 arm_stuck</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>The Lead Arm Remains Connected To The Thorax.</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>리드암이 흉곽에 계속 붙어 있다.</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>Lead Arm Trapped On Chest
 No Arm Separation</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="11" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>The Lead Hip Cannot Accept Body Load.</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>리드 고관절이 하중을 받아들이지 못한다.</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>Lead Hip Fails To Load
 No Left Hip Acceptance</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>early_extension
 pelvis_stall</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>LOD</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>The Lead Hip Cannot Accept Rotational Load.</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>리드 고관절이 회전 하중을 받아주지 못한다.</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr"/>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>lead_pressure_insufficient</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>P6 신규.</t>
-        </is>
-      </c>
+      <c r="F55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -5460,23 +6085,23 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>The Lead Knee And Hip Drift Excessively Toward The Target.</t>
+          <t>The Lead Hip Cannot Accept Rotational Load.</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>리드 무릎과 고관절이 목표 방향으로 과도하게 이동한다.</t>
+          <t>리드 고관절이 회전 하중을 받아주지 못한다.</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr"/>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive</t>
+          <t>lead_pressure_insufficient</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>P6 신규 (프로 지정 핵심 문장). 무릎·고관절·압력 Feature 연결 중간 Mechanism — 향후 재사용 예정.</t>
+          <t>P6 신규.</t>
         </is>
       </c>
     </row>
@@ -5488,304 +6113,502 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
+          <t>The Lead Knee And Hip Drift Excessively Toward The Target.</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>리드 무릎과 고관절이 목표 방향으로 과도하게 이동한다.</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>lead_pressure_excessive</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규 (프로 지정 핵심 문장). 무릎·고관절·압력 Feature 연결 중간 Mechanism — 향후 재사용 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>LOD</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
           <t>The Lead Leg Accepts Body Load Too Early.</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>리드다리가 너무 일찍 하중을 받아낸다.</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Early Lead Leg Load
 Left Leg Loads Too Soon</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>The Lead Side Cannot Stabilize During Transition.</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>전환 과정에서 리드측이 안정되지 못한다.</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>Lead Side Collapses
 No Left Side Stability</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>early_extension</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="F59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>The Trail Side Continues Supporting Rotation.</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>트레일측이 계속 회전을 지지한다.</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>Trail Side Keeps Posting
 Right Side Stays Loaded</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>hanging_back
 head_hanging_back</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="12" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Excessive Trail Side Bend Lowers The Head.</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>과도한 트레일측 측굴로 머리가 낮아진다.</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>head_drop</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Head Drop Side-bend type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>The Arms Compensate For Delayed Body Motion.</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>몸의 지연을 팔이 보상한다.</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr">
         <is>
           <t>Arms Save The Swing
 Arm Compensation</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release
 arm_stuck</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>The Arms Continue Driving Instead Of Rotating Around The Lead Side.</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>리드측 회전 대신 팔 위주의 전달이 이루어진다.</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>Arm Driven Delivery</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>lead_pressure_insufficient</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>P6 신규. Body→Arm driven 전환.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="12" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>The Body Extends Early To Create Space.</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>공간을 만들기 위해 몸이 일찍 신전한다.</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
         <is>
           <t>Stand Up To Make Room
 Early Extension Compensation</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E64" s="4" t="inlineStr">
         <is>
           <t>early_extension
 spine_extension_excessive
 head_elevation</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="12" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>The Hands Take Over Club Delivery.</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>손이 클럽 전달을 주도한다.</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr">
         <is>
           <t>Hand Dominance Increase
 Hands Take Control</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>flip_release
 casting
 hand_dominance_increase</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="12" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>The Head Remains On The Trail Side.</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>머리가 트레일측에 남는다.</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr"/>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>head_hanging_back</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Head 수평축(위치) 링크.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>The Head Rises As The Body Stands Up.</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>몸이 일어나면서 머리가 상승한다.</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr"/>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>head_elevation
+spine_extension_excessive</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Early Extension/Spine → Head Elevation 공통 링크.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>The Lead Arm Separates From The Thorax.</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>리드암이 몸통과 분리된다.</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr">
         <is>
           <t>Chicken Wing
 Lead Arm Flies Off Chest</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr"/>
-      <c r="F64" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>시트 M007. Chicken Wing 전조. P7 연계용 예약.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B65" s="4" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>The Swing Axis Shifts Upward.</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>회전축이 위로 이동한다.</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr"/>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>head_elevation</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>The Torso Extends Backward To Recover Balance.</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>균형 회복을 위해 상체가 뒤로 신전한다.</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr"/>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>spine_extension_excessive
+head_elevation</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Head/Spine 자세 보상 도메인.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>The Torso Flexes Excessively And The Head Drops.</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>상체가 과도하게 굴곡되며 머리가 낮아진다.</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr"/>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>head_drop</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Head Drop Flexion type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>The Trail Arm Extends Early To Deliver The Club.</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>클럽 전달을 위해 트레일 팔이 일찍 펴진다.</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
         <is>
           <t>Right Arm Straightens Early
 Early Trail Arm Extension</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>casting</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="12" t="inlineStr">
+      <c r="F72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>The Trail Elbow Collapses Toward The Body.</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>트레일 팔꿈치가 몸통 쪽으로 급격하게 붙는다.</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D73" s="4" t="inlineStr">
         <is>
           <t>Trail Elbow Pinch
 Right Elbow Jams In</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="E73" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="F73" s="4" t="inlineStr">
         <is>
           <t>시트 M006.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F66"/>
+  <autoFilter ref="A1:F73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5796,7 +6619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6783,8 +7606,148 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Spine Flexion Excessive</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>척추 과굴곡</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 척추(흉요추)가 정상보다 과도하게 굴곡되어 상체가 숙여지는 현상. Spine Extension Excessive와 반대 방향.</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Spine</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Magnitude, Excessive
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Trail Side Bend Excessive</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>트레일측 측굴 과다</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸통의 트레일측 측면 굴곡이 정상보다 과도한 현상.</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Thorax</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Magnitude, Excessive
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Handle Raise</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>핸들 상승</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 그립 핸들이 정상보다 상승하는 현상.</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Shaft</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Motion, Raise
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Handle Too Low</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>핸들 낮음</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 그립 핸들이 정상보다 낮은 위치에 있는 현상.</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Shaft</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Position, Height, Low
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Spine Angle Loss</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>척추각 소실</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 어드레스에서 형성된 척추 전경각이 조기에 소실되는 현상.</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Spine</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Magnitude, Loss
+[status] pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E35"/>
+  <autoFilter ref="A1:E40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6795,7 +7758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6897,346 +7860,358 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>★ 등급</t>
+          <t>현재 표기</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>★★★★★ = 거의 항상 동반 / ★★★★☆ = 매우 자주 동반 (동반 강도 순 정렬)</t>
+          <t>무등급 나열만 유지 (· Feature). 성급한 ★ 부여 금지.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr"/>
-      <c r="B13" s="15" t="inlineStr"/>
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>★ 일괄 부여</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>P6 전 Feature 완료 후 'Co-occurrence Review Day'(Feature 수정 금지, ★ 검토 전용)에 일괄 부여. 예정 등급: ★★★★★ 거의 항상 / ★★★★☆ 매우 자주 / ★★★☆☆ 자주</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr"/>
+      <c r="B14" s="15" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Attribute Vocabulary</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Magnitude</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>Excessive, Insufficient</t>
-        </is>
-      </c>
+      <c r="B15" s="15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Timing</t>
+          <t>Magnitude</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Early, Late</t>
+          <t>Excessive, Insufficient</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Timing</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>Lead, Trail, Heel, Toe</t>
+          <t>Early, Late</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Rotation</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Open, Closed, Stall, Insufficient, Excessive, Early, Late</t>
+          <t>Lead, Trail, Heel, Toe</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Rotation</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>Lift, Drop, Raise, Fall, Rise, Slide, Sway, Push, Pull, Throw</t>
+          <t>Open, Closed, Stall, Insufficient, Excessive, Early, Late</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Position_Height</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>High, Low</t>
+          <t>Lift, Drop, Raise, Fall, Rise, Slide, Sway, Push, Pull, Throw</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>Position_Depth</t>
+          <t>Position_Height</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Deep, Shallow</t>
+          <t>High, Low</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>Position_Width</t>
+          <t>Position_Depth</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>Wide, Close</t>
+          <t>Deep, Shallow</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>Position_Direction</t>
+          <t>Position_Width</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>Forward, Backward, Inside, Outside</t>
+          <t>Wide, Close</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Angle_Plane</t>
+          <t>Position_Direction</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Steep, Flat, Shallow</t>
+          <t>Forward, Backward, Inside, Outside</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>Angle_Axis</t>
+          <t>Angle_Plane</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Vertical, Horizontal</t>
+          <t>Steep, Flat, Shallow</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>ClubFace</t>
+          <t>Angle_Axis</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Open, Closed, Square</t>
+          <t>Vertical, Horizontal</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>Shaft_Orientation</t>
+          <t>ClubFace</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>Stand Up, Lay Down</t>
+          <t>Open, Closed, Square</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Shaft_Orientation</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Early, Late, Flip, Cast</t>
+          <t>Stand Up, Lay Down</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Early, Late, Flip, Cast</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
           <t>Relationship</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Wide, Narrow, Far, Close</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr"/>
-      <c r="B30" s="15" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr"/>
+      <c r="B31" s="15" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Mechanism Categories</t>
         </is>
       </c>
-      <c r="B31" s="15" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>ROT</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="inlineStr">
-        <is>
-          <t>Rotation — 골반/흉곽 회전 (Amount·Timing·Velocity·Axis)</t>
-        </is>
-      </c>
+      <c r="B32" s="15" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>PRS</t>
+          <t>ROT</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Pressure — 트레일/리드 하중 및 압력 이동</t>
+          <t>Rotation — 골반/흉곽 회전 (Amount·Timing·Velocity·Axis)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>PRS</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>Arm Delivery — 팔·손·팔꿈치의 하강과 전달</t>
+          <t>Pressure — 트레일/리드 하중 및 압력 이동</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>CLB</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>Club Delivery — 릴리즈·경로·가파름·최저점·래그</t>
+          <t>Arm Delivery — 팔·손·팔꿈치의 하강과 전달</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>SPC</t>
+          <t>CLB</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>Space — 몸-팔 전달 공간</t>
+          <t>Club Delivery — 릴리즈·경로·가파름·최저점·래그</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>LOD</t>
+          <t>SPC</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
+          <t>Space — 몸-팔 전달 공간</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
+          <t>LOD</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>Compensation — 팔·손·몸의 보상 동작</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr"/>
-      <c r="B39" s="15" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="15" t="inlineStr"/>
+      <c r="B40" s="15" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>Rename Log</t>
         </is>
       </c>
-      <c r="B40" s="15" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>Upper Body Open Early  →  Thorax Open Early</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="inlineStr">
-        <is>
-          <t>해부학 객체명으로 통일 (Upper Body 용어 폐기)</t>
-        </is>
-      </c>
+      <c r="B41" s="15" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>Excessive Spine Extension  →  Spine Extension Excessive</t>
+          <t>Upper Body Open Early  →  Thorax Open Early</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>[Object]+[Attribute] 어순 통일 (Modifier 후치)</t>
+          <t>해부학 객체명으로 통일 (Upper Body 용어 폐기)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
+          <t>Excessive Spine Extension  →  Spine Extension Excessive</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>[Object]+[Attribute] 어순 통일 (Modifier 후치)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
           <t>Upper Body Dominance  →  Body Rotation Dominant</t>
         </is>
       </c>
-      <c r="B43" s="15" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>Upper Body 용어 폐기, cause-side 표준화</t>
         </is>
@@ -7253,7 +8228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7554,14 +8529,14 @@
           <t>Spine Extension Excessive (척추 과신전)</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -7579,14 +8554,14 @@
           <t>Head Elevation (머리 상승)</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -7604,14 +8579,14 @@
           <t>Head Drop (머리 하강)</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -7629,14 +8604,14 @@
           <t>Head Hanging Back (머리 뒤잔류)</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -7998,7 +8973,21 @@
       </c>
     </row>
     <row r="32">
-      <c r="C32" s="22" t="inlineStr">
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>Phase 2-1: 모든 P6 Feature 6섹션 표준화 (진행 중)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>Phase 2-2: Co-occurrence Review Day — 전 Feature 완료 후 Strong Co-occurrence에 ★ 등급 일괄 부여 (그날은 Feature 수정 금지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" s="23" t="inlineStr">
         <is>
           <t>Changelog 메모: 큰 변경은 이 시트 하단에 한 줄씩 기록 (엑셀 바이너리 git diff 불투명성 보완)</t>
         </is>

</xml_diff>

<commit_message>
feat(P6): Hands 5 + Arm 2 + Shaft 2 + Casting 표준화 — Phase 2-1 완료 (28/28)
P6 전 Feature 6섹션 표준화 완료. 이제 Phase 2-2(Co-occurrence Review Day) 준비 완료.

P6 표준화 +10 (6섹션):
  Low/Deep/Forward Hands · Hands Too Far/Too Close · Late Arm
  · Trail Elbow Behind Body · Steep Shaft · Shallow Shaft · Casting
  → 28/28 완료 ✅

Dictionary-first
- 신규 Mechanism 6 (CLB 3·SPC 1·CMP 1·ARM 1) → 총 78
  · 전달 평면(delivery plane)·커넥션·샤프트 뒤처짐·Chicken Wing 링크
  · 나머지는 기존 재사용 (M-ARM/CLB/CMP/SPC/ROT/PRS)
- 신규 Feature 10 (Chicken Wing/Inside Delivery/Over The Top/Trail Elbow Flying
  /Shaft Lay Down/Handle Deep/High AoA/Push Tendency/Impact Consistency/Lead Arm Sep) → 49

핵심 구조 확인
- Steep Shaft = P6 Arm/Club Hub (상류 수렴·하류 분기)
- Shallow Shaft = Good vs Compensation 양면성 명시
- Casting = 같은 결과·다른 메커니즘(Pressure Insuf/Excess) 재확인

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/DOH_Knowledge.xlsx
+++ b/DOH_Knowledge.xlsx
@@ -14,8 +14,8 @@
     <sheet name="TODO" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$73</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TODO'!$A$1:$E$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,11 +67,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00B06A00"/>
+      <color rgb="001F4E5F"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E5F"/>
+      <color rgb="00B06A00"/>
     </font>
     <font>
       <i val="1"/>
@@ -219,11 +219,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -590,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B296"/>
+  <dimension ref="A1:B404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4109,228 +4107,1690 @@
     <row r="269">
       <c r="A269" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 정의</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="271" ht="22" customHeight="1">
-      <c r="A271" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B271" s="2" t="inlineStr">
-        <is>
-          <t>Deep Hands  (손 깊음)   ·   Hands / Position/Depth · Deep</t>
+          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 낮은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 과도하게 하강한 상대 위치가 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B270" s="4" t="inlineStr">
+        <is>
+          <t>Trail Side Bend Excessive (트레일측 측굴 과다)
+   ↓
+Low Hands (손 낮음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="4" t="inlineStr"/>
+      <c r="B271" s="4" t="inlineStr">
+        <is>
+          <t>Head Drop (머리 하강)
+   ↓
+Low Hands (손 낮음)</t>
         </is>
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A272" s="4" t="inlineStr"/>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="274" ht="22" customHeight="1">
-      <c r="A274" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B274" s="2" t="inlineStr">
-        <is>
-          <t>Forward Hands  (손 전방)   ·   Hands / Position/Direction · Forward</t>
+          <t>Shallow Shaft (눕는 샤프트)
+   ↓
+Low Hands (손 낮음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="4" t="inlineStr"/>
+      <c r="B273" s="4" t="inlineStr">
+        <is>
+          <t>Deep Hands (손 깊음)
+   ↓
+Low Hands (손 낮음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="4" t="inlineStr"/>
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t>Handle Too Low (핸들 낮음)
+   ↓
+Low Hands (손 낮음)</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="277" ht="22" customHeight="1">
-      <c r="A277" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B277" s="2" t="inlineStr">
-        <is>
-          <t>Hands Too Far From Body  (손이 몸에서 멀어짐)   ·   Hands / Relationship · Far</t>
+          <t>Low Hands (손 낮음)
+   ↓
+The Club Approaches From Inside.
+(클럽이 안쪽 경로로 접근한다.)
+   ↓
+Inside Delivery (인사이드 딜리버리)</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="4" t="inlineStr"/>
+      <c r="B276" s="4" t="inlineStr">
+        <is>
+          <t>Low Hands (손 낮음)
+   ↓
+Shallow Shaft (눕는 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="4" t="inlineStr"/>
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>Low Hands (손 낮음)
+   ↓
+Deep Hands (손 깊음)</t>
         </is>
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A278" s="4" t="inlineStr"/>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="280" ht="22" customHeight="1">
-      <c r="A280" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B280" s="2" t="inlineStr">
-        <is>
-          <t>Hands Too Close To Body  (손이 몸에 가까움)   ·   Hands / Relationship · Close</t>
+          <t>Low Hands (손 낮음)
+   ↓
+Shaft Lay Down (샤프트 눕힘)</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="4" t="inlineStr"/>
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t>Low Hands (손 낮음)
+   ↓
+Club Face Closed (클럽페이스 클로즈)  ※보상 방식에 따라</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B280" s="4" t="inlineStr">
+        <is>
+          <t>· Shallow Shaft (눕는 샤프트)
+· Shaft Lay Down (샤프트 눕힘)
+· Deep Hands (손 깊음)
+· Head Drop (머리 하강)
+· Trail Side Bend Excessive (트레일측 측굴 과다)
+· Club Face Closed (클럽페이스 클로즈)</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 추가 검증 포인트</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="283" ht="22" customHeight="1">
-      <c r="A283" s="1" t="inlineStr">
+          <t>· High Hands/Low Hands는 절대 좌표가 아니라 다운스윙 진행(골반·흉곽 회전) 대비 상대 위치 Feature.
+· Subtype: Side Bend Type(측굴) / Shallow Type(샤프트 눕힘).</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B282" s="4" t="inlineStr">
+        <is>
+          <t>· P6 손 위치 Feature는 모두 상대 위치(Relative Position): '이 시점 정상이라면 손이 어디 있어야 하는가' 기준. High/Low/Deep/Shallow 동일 철학.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="22" customHeight="1">
+      <c r="A284" s="1" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="B283" s="2" t="inlineStr">
-        <is>
-          <t>Late Arm  (팔 하강 지연)   ·   Arm / Timing · Late</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
-      <c r="B284" s="4" t="inlineStr">
-        <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="286" ht="22" customHeight="1">
-      <c r="A286" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B286" s="2" t="inlineStr">
-        <is>
-          <t>Trail Elbow Behind Body  (트레일 팔꿈치 뒤처짐)   ·   Trail Elbow / Location · Trail</t>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Deep Hands  (손 깊음)   ·   Hands / Position/Depth · Deep</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B285" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽 회전·다운스윙 진행 정도에 비해 손(리드암/그립)이 정상보다 후방에 위치하는 현상. 절대 위치가 아니라 몸통 대비 손이 뒤에 남아있는 상대 위치가 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B286" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Rotation Insufficient (P4, 백스윙 흉곽 회전 부족)
+   ↓
+Lead Arm Depth Insufficient (P4, 리드암 깊이 부족)
+   ↓
+Deep Hands (손 깊음)</t>
         </is>
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A287" s="4" t="inlineStr"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="289" ht="22" customHeight="1">
-      <c r="A289" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B289" s="2" t="inlineStr">
-        <is>
-          <t>Steep Shaft  (가파른 샤프트)   ·   Shaft / Angle/Plane · Steep</t>
+          <t>Arm Drop Insufficient (팔 하강 부족)
+   ↓
+Vertical Arm Drop During Downswing Is Insufficient.
+(다운스윙 동안 팔의 수직 하강이 충분하지 않다.)
+   ↓
+Deep Hands (손 깊음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="4" t="inlineStr"/>
+      <c r="B288" s="4" t="inlineStr">
+        <is>
+          <t>Trail Elbow Stuck (트레일 팔꿈치 끼임)
+   ↓
+The Trail Elbow Collapses Toward The Body.
+(트레일 팔꿈치가 몸통 쪽으로 급격하게 붙는다.)
+   ↓
+Deep Hands (손 깊음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="4" t="inlineStr"/>
+      <c r="B289" s="4" t="inlineStr">
+        <is>
+          <t>Arm Depth Excessive (P4, 백스윙 손 과도한 깊이)
+   ↓
+The Hands Start Downswing From Behind The Thorax.
+(손이 몸통보다 뒤쪽에서 다운스윙을 시작한다.)
+   ↓
+Deep Hands (손 깊음)</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 이후 나타날 가능성</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="292" ht="22" customHeight="1">
-      <c r="A292" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B292" s="2" t="inlineStr">
-        <is>
-          <t>Shallow Shaft  (눕는 샤프트)   ·   Shaft / Angle/Plane · Shallow</t>
+          <t>Deep Hands (손 깊음)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Arm Stuck (팔 끼임)
+   ↓
+Late Release (늦은 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="4" t="inlineStr"/>
+      <c r="B291" s="4" t="inlineStr">
+        <is>
+          <t>Deep Hands (손 깊음)
+   ↓
+The Club Approaches From Inside.
+(클럽이 안쪽 경로로 접근한다.)
+   ↓
+Inside Delivery (인사이드 딜리버리)</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="4" t="inlineStr"/>
+      <c r="B292" s="4" t="inlineStr">
+        <is>
+          <t>Deep Hands (손 깊음)
+   ↓
+The Shaft Falls Behind The Hands.
+(샤프트가 손보다 뒤로 떨어진다.)
+   ↓
+Shallow Shaft (눕는 샤프트)</t>
         </is>
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="3" t="inlineStr">
-        <is>
-          <t>(상태)</t>
-        </is>
-      </c>
+      <c r="A293" s="4" t="inlineStr"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="295" ht="22" customHeight="1">
-      <c r="A295" s="1" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="B295" s="2" t="inlineStr">
-        <is>
-          <t>Casting  (캐스팅)   ·   Club / Release · Cast</t>
+          <t>Deep Hands (손 깊음)
+   ↓
+Handle Deep (핸들 깊음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="4" t="inlineStr"/>
+      <c r="B294" s="4" t="inlineStr">
+        <is>
+          <t>Deep Hands (손 깊음)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B295" s="4" t="inlineStr">
+        <is>
+          <t>· Arm Drop Insufficient (팔 하강 부족)
+· Arm Stuck (팔 끼임)
+· Late Release (늦은 릴리즈)
+· Shallow Shaft (눕는 샤프트)
+· Shaft Lay Down (샤프트 눕힘)</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="3" t="inlineStr">
         <is>
-          <t>(상태)</t>
+          <t>■ 추가 검증 포인트</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>표준화 예정 — 원본 P6 기준 순차 진행 (6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence / 추가 검증 포인트 / 사고확장)</t>
+          <t>· Deep Hands는 Hand Feature가 아니라 Relative Feature(몸통 대비 후방).
+· P4 기원(Arm Depth Excessive / Lead Arm Depth Insufficient)이 많음 → P4 시트 연계.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B297" s="4" t="inlineStr">
+        <is>
+          <t>· 관찰 기준(Object Reference)은 흉곽 회전·다운스윙 진행. Deep/Shallow는 몸통 대비 전후 위치 상대 평가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="22" customHeight="1">
+      <c r="A299" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>Forward Hands  (손 전방)   ·   Hands / Position/Direction · Forward</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B300" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽 회전·다운스윙 진행 정도에 비해 손(리드암/그립)이 정상보다 몸의 전방에 위치하는 현상. 절대 위치가 아니라 몸통 대비 손이 앞서 있는 상대 위치가 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B301" s="4" t="inlineStr">
+        <is>
+          <t>Lead Arm Separation Increase (리드암-흉곽 분리 증가)
+   ↓
+Forward Hands (손 전방)</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="4" t="inlineStr"/>
+      <c r="B302" s="4" t="inlineStr">
+        <is>
+          <t>Arm Lift Excessive (P4, 팔 과도한 상승)
+   ↓
+The Arm Starts Downswing From A Higher Position.
+(팔이 높은 위치에서 다운스윙을 시작한다.)
+   ↓
+Vertical Arm Drop During Downswing Is Insufficient.
+(다운스윙 동안 팔의 수직 하강이 충분하지 않다.)
+   ↓
+Forward Hands (손 전방)</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="4" t="inlineStr"/>
+      <c r="B303" s="4" t="inlineStr">
+        <is>
+          <t>Trail Elbow Flying (플라잉 엘보)
+   ↓
+Forward Hands (손 전방)</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="4" t="inlineStr"/>
+      <c r="B304" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트)
+   ↓
+Forward Hands (손 전방)</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B305" s="4" t="inlineStr">
+        <is>
+          <t>Forward Hands (손 전방)
+   ↓
+The Hands Move Ahead Of The Delivery Plane.
+(손이 전달 평면보다 앞쪽에서 이동한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="4" t="inlineStr"/>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t>Forward Hands (손 전방)
+   ↓
+The Club Approaches From Outside.
+(클럽이 바깥쪽 경로로 접근한다.)
+   ↓
+Over The Top (오버 더 탑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="4" t="inlineStr"/>
+      <c r="B307" s="4" t="inlineStr">
+        <is>
+          <t>Forward Hands (손 전방)
+   ↓
+Outside Delivery (아웃사이드 딜리버리)</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="4" t="inlineStr"/>
+      <c r="B308" s="4" t="inlineStr">
+        <is>
+          <t>Forward Hands (손 전방)
+   ↓
+High Hands (손 높음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B309" s="4" t="inlineStr">
+        <is>
+          <t>· High Hands (손 높음)
+· Steep Shaft (가파른 샤프트)
+· Over The Top (오버 더 탑)
+· Outside Delivery (아웃사이드 딜리버리)
+· Trail Elbow Flying (플라잉 엘보)</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B310" s="4" t="inlineStr">
+        <is>
+          <t>· Forward Hands와 High Hands의 선후 관계 검증 (둘 다 Steep/OTT 상류).</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B311" s="4" t="inlineStr">
+        <is>
+          <t>· 손의 전후(Depth) 축: Deep(후방) ↔ Forward(전방). 몸통 대비 상대 위치로 관리.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="22" customHeight="1">
+      <c r="A313" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>Hands Too Far From Body  (손이 몸에서 멀어짐)   ·   Hands / Relationship · Far</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B314" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸통 회전·다운스윙 진행 정도에 비해 양손이 정상보다 몸통에서 멀리 위치하는 현상. 절대 위치가 아니라 양팔(특히 트레일 팔)이 몸통과의 커넥션(Connection)을 충분히 유지하지 못한 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B315" s="4" t="inlineStr">
+        <is>
+          <t>Trail Elbow Flying (플라잉 엘보)
+   ↓
+The Trail Arm Loses Connection With The Thorax.
+(트레일 팔이 몸통과의 커넥션을 잃는다.)
+   ↓
+Hands Too Far From Body (손이 몸에서 멀어짐)</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="4" t="inlineStr"/>
+      <c r="B316" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive (리드측 압력 과다)
+   ↓
+The Body Reaches The Lead Side Before The Arms.
+(몸이 팔보다 먼저 리드측에 도달한다.)
+   ↓
+Hands Too Far From Body (손이 몸에서 멀어짐)</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="4" t="inlineStr"/>
+      <c r="B317" s="4" t="inlineStr">
+        <is>
+          <t>Backswing Trail Arm Connection Loss (백스윙 트레일 팔 커넥션 상실)
+   ↓
+Hands Too Far From Body (손이 몸에서 멀어짐)</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B318" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Far From Body (손이 몸에서 멀어짐)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="4" t="inlineStr"/>
+      <c r="B319" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Far From Body (손이 몸에서 멀어짐)
+   ↓
+The Club Approaches From Outside.
+(클럽이 바깥쪽 경로로 접근한다.)
+   ↓
+Over The Top (오버 더 탑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="4" t="inlineStr"/>
+      <c r="B320" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Far From Body (손이 몸에서 멀어짐)
+   ↓
+The Club Is Released Early To Reach The Ball.
+(공에 도달하기 위해 클럽을 조기에 푼다.)
+   ↓
+Early Release (이른 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B321" s="4" t="inlineStr">
+        <is>
+          <t>· Trail Elbow Flying (플라잉 엘보)
+· Early Release (이른 릴리즈)
+· Steep Shaft (가파른 샤프트)
+· Over The Top (오버 더 탑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B322" s="4" t="inlineStr">
+        <is>
+          <t>· 몸통과 팔의 커넥션(Connection) 유지 실패가 본질 — 백스윙 기원(P4) 여부 검증.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B323" s="4" t="inlineStr">
+        <is>
+          <t>· Hands 위치는 Height(High/Low)·Depth(Deep/Forward)·Relationship(Far/Close) 세 축으로 관리. Far/Close는 커넥션(Arm Space) 축.</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="22" customHeight="1">
+      <c r="A325" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body  (손이 몸에 가까움)   ·   Hands / Relationship · Close</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B326" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸통 회전·다운스윙 진행 정도에 비해 양손이 정상보다 몸통에 과도하게 가까이 위치하는 현상. 손과 몸통 사이의 공간(Arm Space)이 부족한 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B327" s="4" t="inlineStr">
+        <is>
+          <t>Trail Elbow Stuck (트레일 팔꿈치 끼임)
+   ↓
+The Trail Arm Folds Excessively Toward The Thorax.
+(트레일 팔이 몸통 쪽으로 과도하게 접힌다.)
+   ↓
+Hands Too Close To Body (손이 몸에 가까움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="4" t="inlineStr"/>
+      <c r="B328" s="4" t="inlineStr">
+        <is>
+          <t>Deep Hands (손 깊음)
+   ↓
+Hands Too Close To Body (손이 몸에 가까움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B329" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body (손이 몸에 가까움)
+   ↓
+The Club Approaches From Inside.
+(클럽이 안쪽 경로로 접근한다.)
+   ↓
+Inside Delivery (인사이드 딜리버리)</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="4" t="inlineStr"/>
+      <c r="B330" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body (손이 몸에 가까움)
+   ↓
+Arm Delivery Space Is Reduced.
+(팔이 내려올 공간이 감소한다.)
+   ↓
+Early Release (이른 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="4" t="inlineStr"/>
+      <c r="B331" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body (손이 몸에 가까움)
+   ↓
+The Lead Arm Cannot Extend Through Impact.
+(리드암이 임팩트 구간에서 충분히 뻗지 못한다.)
+   ↓
+Chicken Wing Pattern (치킨윙 패턴)</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="4" t="inlineStr"/>
+      <c r="B332" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body (손이 몸에 가까움)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
+Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="4" t="inlineStr"/>
+      <c r="B333" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body (손이 몸에 가까움)
+   ↓
+Arm Delivery Space Is Reduced.
+(팔이 내려올 공간이 감소한다.)
+   ↓
+Arm Stuck (팔 끼임)</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B334" s="4" t="inlineStr">
+        <is>
+          <t>· Trail Elbow Stuck (트레일 팔꿈치 끼임)
+· Deep Hands (손 깊음)
+· Shallow Shaft (눕는 샤프트)
+· Inside Delivery (인사이드 딜리버리)
+· Early Release (이른 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B335" s="4" t="inlineStr">
+        <is>
+          <t>· Arm Space 부족이 Early Extension/Chicken Wing 중 어느 보상으로 가는지 Subtype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B336" s="4" t="inlineStr">
+        <is>
+          <t>· Hands Too Close는 Arm Space 부족의 대표 신호 — Early Extension(공간 확보 보상)의 주요 상류.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="22" customHeight="1">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>Late Arm  (팔 하강 지연)   ·   Arm / Timing · Late</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B339" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸통 회전·다운스윙 진행 정도에 비해 팔의 하강이 정상보다 늦은 현상. 팔 자체 속도가 느린 것이 아니라 몸통 대비 팔이 상대적으로 늦게 전달되는 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B340" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
+   ↓
+Thorax Rotation Outpaces Arm Delivery.
+(흉곽 회전이 팔 전달보다 앞선다.)
+   ↓
+Late Arm (팔 하강 지연)</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="4" t="inlineStr"/>
+      <c r="B341" s="4" t="inlineStr">
+        <is>
+          <t>Early Pressure Shift (조기 압력 이동)
+   ↓
+The Body Reaches The Lead Side Before The Arms.
+(몸이 팔보다 먼저 리드측에 도달한다.)
+   ↓
+Late Arm (팔 하강 지연)</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="4" t="inlineStr"/>
+      <c r="B342" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Open Early (골반 조기 오픈)
+   ↓
+The Pelvis Rotates Faster Than The Arms Can Follow.
+(팔이 따라올 수 없을 만큼 골반이 빠르게 회전한다.)
+   ↓
+Late Arm (팔 하강 지연)</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="4" t="inlineStr"/>
+      <c r="B343" s="4" t="inlineStr">
+        <is>
+          <t>Arm Depth Excessive (P4, 백스윙 손 과도한 깊이)
+   ↓
+The Hands Start Downswing From Behind The Thorax.
+(손이 몸통보다 뒤쪽에서 다운스윙을 시작한다.)
+   ↓
+Rapid Thorax Rotation Reduces Available Arm Drop Time.
+(급격한 흉곽 회전으로 팔이 하강할 시간이 부족해진다.)
+   ↓
+Late Arm (팔 하강 지연)</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B344" s="4" t="inlineStr">
+        <is>
+          <t>Late Arm (팔 하강 지연)
+   ↓
+The Hands Remain Above The Delivery Plane.
+(손이 전달 평면보다 높은 위치를 유지한다.)
+   ↓
+High Hands (손 높음)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="4" t="inlineStr"/>
+      <c r="B345" s="4" t="inlineStr">
+        <is>
+          <t>Late Arm (팔 하강 지연)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+Arm Stuck (팔 끼임)</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="4" t="inlineStr"/>
+      <c r="B346" s="4" t="inlineStr">
+        <is>
+          <t>Late Arm (팔 하강 지연)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B347" s="4" t="inlineStr">
+        <is>
+          <t>· High Hands (손 높음)
+· Steep Shaft (가파른 샤프트)
+· Arm Stuck (팔 끼임)
+· Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)
+· Over The Top (오버 더 탑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B348" s="4" t="inlineStr">
+        <is>
+          <t>· Late Arm은 Rotation Type / Pressure Type / P4 Type 세 갈래 — 원인 Type을 함께 기록.</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B349" s="4" t="inlineStr">
+        <is>
+          <t>· Late Arm은 몸통-팔 시퀀스 붕괴의 핵심 관측 지표. Thorax/Pelvis Open Early·Early Pressure Shift의 공통 하류이자 High Hands/Steep Shaft의 상류.</t>
+        </is>
+      </c>
+    </row>
+    <row r="351" ht="22" customHeight="1">
+      <c r="A351" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B351" s="2" t="inlineStr">
+        <is>
+          <t>Trail Elbow Behind Body  (트레일 팔꿈치 뒤처짐)   ·   Trail Elbow / Location · Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B352" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸통 회전·다운스윙 진행 정도에 비해 트레일 팔꿈치가 정상보다 몸통의 후방에 위치하는 현상. 절대 위치가 아니라 몸통 대비 트레일 팔꿈치가 뒤에 남아있는 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B353" s="4" t="inlineStr">
+        <is>
+          <t>Late Arm (팔 하강 지연)
+   ↓
+Thorax Rotation Outpaces Arm Delivery.
+(흉곽 회전이 팔 전달보다 앞선다.)
+   ↓
+The Trail Elbow Falls Behind The Thorax.
+(트레일 팔꿈치가 흉곽보다 뒤처진다.)
+   ↓
+Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B354" s="4" t="inlineStr">
+        <is>
+          <t>Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)
+   ↓
+The Trail Arm Extends Early To Deliver The Club.
+(클럽 전달을 위해 트레일 팔이 일찍 펴진다.)
+   ↓
+High Angle Of Attack (높은 어택앵글)</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="4" t="inlineStr"/>
+      <c r="B355" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트) + Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)
+   ↓
+The Lead Arm Cannot Extend Through Impact.
+(리드암이 임팩트 구간에서 충분히 뻗지 못한다.)
+   ↓
+Chicken Wing Pattern (치킨윙 패턴)</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="4" t="inlineStr"/>
+      <c r="B356" s="4" t="inlineStr">
+        <is>
+          <t>Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)
+   ↓
+The Trail Elbow Collapses Toward The Body.
+(트레일 팔꿈치가 몸통 쪽으로 급격하게 붙는다.)
+   ↓
+The Shaft Falls Behind The Hands.
+(샤프트가 손보다 뒤로 떨어진다.)
+   ↓
+Shallow Shaft (눕는 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B357" s="4" t="inlineStr">
+        <is>
+          <t>· Late Arm (팔 하강 지연)
+· Arm Stuck (팔 끼임)
+· Steep Shaft (가파른 샤프트)
+· Chicken Wing Pattern (치킨윙 패턴)
+· Shallow Shaft (눕는 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B358" s="4" t="inlineStr">
+        <is>
+          <t>· Trail Elbow Behind Body → Steep(급격 신전, 부하↑) vs Shallow(급격 붙음) 두 분기 — 어느 쪽이 더 흔한지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B359" s="4" t="inlineStr">
+        <is>
+          <t>· 몸통 대비 트레일 팔꿈치 후방. Chicken Wing·High AoA·관절 부하 증가로 이어지는 상해 위험 경로의 상류.</t>
+        </is>
+      </c>
+    </row>
+    <row r="361" ht="22" customHeight="1">
+      <c r="A361" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B361" s="2" t="inlineStr">
+        <is>
+          <t>Steep Shaft  (가파른 샤프트)   ·   Shaft / Angle/Plane · Steep</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B362" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 가파른 현상. 손·클럽이 전달 평면보다 위 또는 바깥에서 접근하는 것이 핵심이다. 다수 상류가 수렴하고 다수 하류로 분기하는 Hub 성격.</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B363" s="4" t="inlineStr">
+        <is>
+          <t>High Hands (손 높음)
+   ↓
+The Hands Remain Above The Delivery Plane.
+(손이 전달 평면보다 높은 위치를 유지한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="4" t="inlineStr"/>
+      <c r="B364" s="4" t="inlineStr">
+        <is>
+          <t>Late Arm (팔 하강 지연)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+High Hands (손 높음)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="4" t="inlineStr"/>
+      <c r="B365" s="4" t="inlineStr">
+        <is>
+          <t>Forward Hands (손 전방)
+   ↓
+The Hands Move Ahead Of The Delivery Plane.
+(손이 전달 평면보다 앞쪽에서 이동한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="4" t="inlineStr"/>
+      <c r="B366" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Far From Body (손이 몸에서 멀어짐)
+   ↓
+The Club Approaches From Outside.
+(클럽이 바깥쪽 경로로 접근한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="4" t="inlineStr"/>
+      <c r="B367" s="4" t="inlineStr">
+        <is>
+          <t>Thorax Open Early (흉곽 조기 오픈)
+   ↓
+Thorax Rotation Outpaces Arm Delivery.
+(흉곽 회전이 팔 전달보다 앞선다.)
+   ↓
+Late Arm (팔 하강 지연)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B368" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트)
+   ↓
+The Clubhead Travels More Vertically Into Impact.
+(클럽헤드가 더욱 수직에 가까운 경로로 임팩트에 접근한다.)
+   ↓
+High Angle Of Attack (높은 어택앵글)</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="4" t="inlineStr"/>
+      <c r="B369" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트)
+   ↓
+The Lead Arm Cannot Extend Through Impact.
+(리드암이 임팩트 구간에서 충분히 뻗지 못한다.)
+   ↓
+Chicken Wing Pattern (치킨윙 패턴)</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="4" t="inlineStr"/>
+      <c r="B370" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
+Early Extension (얼리 익스텐션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="4" t="inlineStr"/>
+      <c r="B371" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트)
+   ↓
+The Body Extends Early To Create Space.
+(공간을 만들기 위해 몸이 일찍 신전한다.)
+   ↓
+Head Elevation (머리 상승)</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="4" t="inlineStr"/>
+      <c r="B372" s="4" t="inlineStr">
+        <is>
+          <t>Steep Shaft (가파른 샤프트)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B373" s="4" t="inlineStr">
+        <is>
+          <t>· High Hands (손 높음)
+· Forward Hands (손 전방)
+· Over The Top (오버 더 탑)
+· Outside Delivery (아웃사이드 딜리버리)
+· Early Extension (얼리 익스텐션)
+· Chicken Wing Pattern (치킨윙 패턴)</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B374" s="4" t="inlineStr">
+        <is>
+          <t>· Steep Shaft 상류 Type(High Hands/Late Arm/Forward Hands/OTT/Thorax Open Early) 중 어느 경로가 가장 흔한지 (Co-occurrence Review Day에서 ★).</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B375" s="4" t="inlineStr">
+        <is>
+          <t>· Steep Shaft는 P6 Arm/Club 계열의 대표 Hub — 상류 다수 수렴, 하류(AoA↑/Chicken Wing/Early Extension/Flip)로 분기. 상해 부하(팔꿈치·손목) 경로의 관문.</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="22" customHeight="1">
+      <c r="A377" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B377" s="2" t="inlineStr">
+        <is>
+          <t>Shallow Shaft  (눕는 샤프트)   ·   Shaft / Angle/Plane · Shallow</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B378" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 눕는 현상. 회전·커넥션이 유지된 Good Shallow와 Laid-off·트레일 붕괴·커넥션 상실에서 나오는 Compensation Shallow를 구분해야 한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B379" s="4" t="inlineStr">
+        <is>
+          <t>Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)
+   ↓
+The Trail Elbow Collapses Toward The Body.
+(트레일 팔꿈치가 몸통 쪽으로 급격하게 붙는다.)
+   ↓
+The Shaft Falls Behind The Hands.
+(샤프트가 손보다 뒤로 떨어진다.)
+   ↓
+Shallow Shaft (눕는 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="4" t="inlineStr"/>
+      <c r="B380" s="4" t="inlineStr">
+        <is>
+          <t>Deep Hands (손 깊음)
+   ↓
+The Club Approaches From Inside.
+(클럽이 안쪽 경로로 접근한다.)
+   ↓
+Shallow Shaft (눕는 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="4" t="inlineStr"/>
+      <c r="B381" s="4" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body (손이 몸에 가까움)
+   ↓
+Arm Delivery Space Is Reduced.
+(팔이 내려올 공간이 감소한다.)
+   ↓
+Shallow Shaft (눕는 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="4" t="inlineStr"/>
+      <c r="B382" s="4" t="inlineStr">
+        <is>
+          <t>Late Arm (팔 하강 지연)
+   ↓
+The Arms Fall Behind The Rotating Body.
+(회전하는 몸에 비해 팔이 뒤처진다.)
+   ↓
+The Shaft Falls Behind The Hands.
+(샤프트가 손보다 뒤로 떨어진다.)
+   ↓
+Shallow Shaft (눕는 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B383" s="4" t="inlineStr">
+        <is>
+          <t>Shallow Shaft (눕는 샤프트)
+   ↓
+The Club Approaches From Inside.
+(클럽이 안쪽 경로로 접근한다.)
+   ↓
+Deep Hands (손 깊음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="4" t="inlineStr"/>
+      <c r="B384" s="4" t="inlineStr">
+        <is>
+          <t>Shallow Shaft (눕는 샤프트)
+   ↓
+Hands Too Close To Body (손이 몸에 가까움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="4" t="inlineStr"/>
+      <c r="B385" s="4" t="inlineStr">
+        <is>
+          <t>Shallow Shaft (눕는 샤프트)
+   ↓
+The Club Approaches From Inside.
+(클럽이 안쪽 경로로 접근한다.)
+   ↓
+Inside Delivery (인사이드 딜리버리)</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="4" t="inlineStr"/>
+      <c r="B386" s="4" t="inlineStr">
+        <is>
+          <t>Shallow Shaft (눕는 샤프트)
+   ↓
+Push Tendency (푸시 경향)</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="4" t="inlineStr"/>
+      <c r="B387" s="4" t="inlineStr">
+        <is>
+          <t>Shallow Shaft (눕는 샤프트)
+   ↓
+Impact Consistency Decrease (임팩트 일관성 감소)</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B388" s="4" t="inlineStr">
+        <is>
+          <t>· Deep Hands (손 깊음)
+· Shaft Lay Down (샤프트 눕힘)
+· Hands Too Close To Body (손이 몸에 가까움)
+· Inside Delivery (인사이드 딜리버리)
+· Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B389" s="4" t="inlineStr">
+        <is>
+          <t>· Good Shallow(회전+커넥션 유지→효율 전달) vs Compensation Shallow(Laid-off/트레일 붕괴/Hands Too Close→타이밍 의존) 반드시 분리.</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B390" s="4" t="inlineStr">
+        <is>
+          <t>· Shallow Shaft는 양면성 Feature — 동일 관찰이 효율 전달일 수도 보상 전달일 수도 있어, 동반 Feature로 Good/Compensation을 판별한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="22" customHeight="1">
+      <c r="A392" s="1" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t>Casting  (캐스팅)   ·   Club / Release · Cast</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="3" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B393" s="4" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 클럽과 리드암 사이의 각도(Lag)가 정상보다 이른 시점에 감소하는 현상. 손목을 의도적으로 푸는 것이 아니라 클럽이 손보다 먼저 풀리기 시작하는 것이 핵심이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="3" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B394" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient (리드측 압력 부족)
+   ↓
+The Arms Continue Driving Instead Of Rotating Around The Lead Side.
+(리드측 회전 대신 팔 위주의 전달이 이루어진다.)
+   ↓
+Casting (캐스팅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="4" t="inlineStr"/>
+      <c r="B395" s="4" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive (리드측 압력 과다)
+   ↓
+The Body Reaches The Lead Side Before The Arms.
+(몸이 팔보다 먼저 리드측에 도달한다.)
+   ↓
+The Club Is Released Early To Reach The Ball.
+(공에 도달하기 위해 클럽을 조기에 푼다.)
+   ↓
+Casting (캐스팅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="4" t="inlineStr"/>
+      <c r="B396" s="4" t="inlineStr">
+        <is>
+          <t>Incomplete Pressure Transfer (압력 이동 미완성)
+   ↓
+The Arms Compensate For Delayed Body Motion.
+(몸의 지연을 팔이 보상한다.)
+   ↓
+Casting (캐스팅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="4" t="inlineStr"/>
+      <c r="B397" s="4" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation Insufficient (골반 회전 부족)
+   ↓
+The Arms Compensate For Delayed Body Motion.
+(몸의 지연을 팔이 보상한다.)
+   ↓
+Casting (캐스팅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="3" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B398" s="4" t="inlineStr">
+        <is>
+          <t>Casting (캐스팅)
+   ↓
+Lag Is Lost Before Impact.
+(임팩트 전에 래그가 소실된다.)
+   ↓
+Loss of Power (파워 손실)</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="4" t="inlineStr"/>
+      <c r="B399" s="4" t="inlineStr">
+        <is>
+          <t>Casting (캐스팅)
+   ↓
+The Clubhead Overtakes The Hands Early.
+(클럽헤드가 손보다 먼저 앞선다.)
+   ↓
+Flip Release (플립 릴리즈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="4" t="inlineStr"/>
+      <c r="B400" s="4" t="inlineStr">
+        <is>
+          <t>Casting (캐스팅)
+   ↓
+The Club Approaches From A Steeper Delivery Pattern.
+(클럽이 가파른 전달 패턴으로 접근한다.)
+   ↓
+Steep Shaft (가파른 샤프트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="4" t="inlineStr"/>
+      <c r="B401" s="4" t="inlineStr">
+        <is>
+          <t>Casting (캐스팅)
+   ↓
+The Club Bottoms Out Behind The Ball.
+(클럽 최저점이 볼 뒤에서 형성된다.)
+   ↓
+Fat Contact (뒤땅)</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="3" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B402" s="4" t="inlineStr">
+        <is>
+          <t>· Lead Pressure Insufficient (리드측 압력 부족)
+· Lead Pressure Excessive (리드측 압력 과다)
+· Incomplete Pressure Transfer (압력 이동 미완성)
+· Flip Release (플립 릴리즈)
+· Loss of Power (파워 손실)</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="3" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B403" s="4" t="inlineStr">
+        <is>
+          <t>· 같은 Casting이라도 원인이 다르다: Lead Pressure Insufficient=공에 도달하려 캐스팅 / Lead Pressure Excessive=몸이 앞서 타이밍 맞추려 캐스팅. 같은 결과·다른 메커니즘 구분이 DOH 핵심 가치.</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B404" s="4" t="inlineStr">
+        <is>
+          <t>· Casting은 Pressure/Rotation 실패의 공통 하류 보상. 정의 기준은 Lag의 조기 소실.</t>
         </is>
       </c>
     </row>
@@ -4345,7 +5805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5569,290 +7029,318 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
+          <t>The Trail Arm Folds Excessively Toward The Thorax.</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>트레일 팔이 몸통 쪽으로 과도하게 접힌다.</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>hands_too_close_to_body</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
           <t>The Trail Elbow Falls Behind The Thorax.</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>트레일 팔꿈치가 흉곽보다 뒤처진다.</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Trail Elbow Stuck
 Right Elbow Behind Body</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Thorax Rotation Outpaces Arm Delivery.</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>흉곽 회전이 팔 전달보다 앞선다.</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>The Chest Beats The Arms
 Body Ahead Of Arms</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>thorax_open_early
 thorax_rotation_excessive</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Vertical Arm Drop During Downswing Is Insufficient.</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>다운스윙 동안 팔의 수직 하강이 충분하지 않다.</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Insufficient Vertical Arm Drop During Downswing</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>high_hands
 steep_shaft</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>시트 M002. M-ARM-06의 수직 방향 특화 변형.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Lag Is Lost Before Impact.</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>임팩트 전에 래그가 소실된다.</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>Loss Of Lag
 Angle Released Too Soon</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>The Club Approaches From A Steeper Delivery Pattern.</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>클럽이 가파른 전달 패턴으로 접근한다.</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>Steep Shaft Delivery
 The Shaft Steepens</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>steep_shaft
 high_hands</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>The Club Approaches From Inside.</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>클럽이 안쪽 경로로 접근한다.</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>Inside Delivery</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>head_drop
 shallow_shaft</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>P6 신규. M-CLB-02(Outside)의 대응 링크.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>The Club Approaches From Outside.</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>클럽이 바깥쪽 경로로 접근한다.</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Over The Top
 Outside Delivery
 Out-To-In Path</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>outside_delivery</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>The Club Bottoms Out Behind The Ball.</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>클럽 최저점이 볼 뒤에서 형성된다.</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>Low Point Behind Ball
 Bottoms Out Early</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>fat_contact
 head_drop
 head_hanging_back</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>The Club Face Cannot Square In Time.</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>클럽페이스가 제시간에 스퀘어되지 못한다.</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>Face Stays Open
 Face Cannot Rotate In Time</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>club_face_open</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>The Club Is Released Early To Reach The Ball.</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>공에 도달하기 위해 클럽을 조기에 푼다.</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Casting
 Early Release
@@ -5860,755 +7348,913 @@
 Hand Dominance Release</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="9" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
         <is>
           <t>CLB</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>The Clubhead Overtakes The Hands Early.</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>클럽헤드가 손보다 먼저 앞선다.</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>Flip
 Clubhead Passes Hands Early
 Scoop</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>flip_release</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>The Hands Move Ahead Of The Delivery Plane.</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>손이 전달 평면보다 앞쪽에서 이동한다.</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>forward_hands
+steep_shaft</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>The Hands Remain Above The Delivery Plane.</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>손이 전달 평면보다 높은 위치를 유지한다.</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>high_hands
+late_arm
+steep_shaft</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Steep Shaft 상류 공통 링크.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>The Shaft Falls Behind The Hands.</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>샤프트가 손보다 뒤로 떨어진다.</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Shaft Falls Behind Body</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>shallow_shaft
+trail_elbow_behind_body</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Shallow Shaft 핵심 링크.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Reduced Arm Space Promotes Early Club Release.</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>팔 공간 부족으로 클럽을 조기에 풀게 된다.</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>No Space Forces Casting
 Tight Space Causes Early Release</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>casting
 early_extension</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="10" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>The Body Loses Delivery Space.</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>다운스윙 공간이 부족해진다.</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>No Room To Deliver
 Space Collapses</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>early_extension
 high_hands</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>The Body Moves Toward The Ball And Loses Space.</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>몸이 볼 방향으로 이동하며 공간을 잃는다.</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>Body Drifts To The Ball
 Toward-Ball Movement</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>early_extension
 high_hands</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>The Body Reaches The Lead Side Before The Arms.</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>몸이 팔보다 먼저 리드측에 도달한다.</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>Body Ahead Of Arms Into Impact
 Body Gets Left First</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early
 arm_stuck</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t>SPC</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>The Lead Arm Remains Connected To The Thorax.</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>리드암이 흉곽에 계속 붙어 있다.</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Lead Arm Trapped On Chest
 No Arm Separation</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>SPC</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>The Trail Arm Loses Connection With The Thorax.</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>트레일 팔이 몸통과의 커넥션을 잃는다.</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Trail Arm Connection Loss</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>hands_too_far_from_body</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Connection 개념.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>The Lead Hip Cannot Accept Body Load.</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>리드 고관절이 하중을 받아들이지 못한다.</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>Lead Hip Fails To Load
 No Left Hip Acceptance</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>early_extension
 pelvis_stall</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="11" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>The Lead Hip Cannot Accept Rotational Load.</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>리드 고관절이 회전 하중을 받아주지 못한다.</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr"/>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr">
         <is>
           <t>lead_pressure_insufficient</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>P6 신규.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>The Lead Knee And Hip Drift Excessively Toward The Target.</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>리드 무릎과 고관절이 목표 방향으로 과도하게 이동한다.</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr"/>
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t>lead_pressure_excessive</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr">
         <is>
           <t>P6 신규 (프로 지정 핵심 문장). 무릎·고관절·압력 Feature 연결 중간 Mechanism — 향후 재사용 예정.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>The Lead Leg Accepts Body Load Too Early.</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>리드다리가 너무 일찍 하중을 받아낸다.</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>Early Lead Leg Load
 Left Leg Loads Too Soon</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>pelvis_open_early</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>The Lead Side Cannot Stabilize During Transition.</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>전환 과정에서 리드측이 안정되지 못한다.</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
         <is>
           <t>Lead Side Collapses
 No Left Side Stability</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="E64" s="4" t="inlineStr">
         <is>
           <t>early_extension</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
         <is>
           <t>LOD</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>The Trail Side Continues Supporting Rotation.</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>트레일측이 계속 회전을 지지한다.</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr">
         <is>
           <t>Trail Side Keeps Posting
 Right Side Stays Loaded</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>hanging_back
 head_hanging_back</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>Excessive Trail Side Bend Lowers The Head.</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>과도한 트레일측 측굴로 머리가 낮아진다.</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr"/>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr"/>
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>head_drop</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>P6 신규. Head Drop Side-bend type.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="12" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>The Arms Compensate For Delayed Body Motion.</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>몸의 지연을 팔이 보상한다.</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t>Arms Save The Swing
 Arm Compensation</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E67" s="4" t="inlineStr">
         <is>
           <t>casting
 flip_release
 arm_stuck</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="12" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>The Arms Continue Driving Instead Of Rotating Around The Lead Side.</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>리드측 회전 대신 팔 위주의 전달이 이루어진다.</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr">
         <is>
           <t>Arm Driven Delivery</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t>lead_pressure_insufficient</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>P6 신규. Body→Arm driven 전환.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="12" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>The Body Extends Early To Create Space.</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>공간을 만들기 위해 몸이 일찍 신전한다.</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
         <is>
           <t>Stand Up To Make Room
 Early Extension Compensation</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>early_extension
 spine_extension_excessive
 head_elevation</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="12" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B65" s="4" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>The Hands Take Over Club Delivery.</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>손이 클럽 전달을 주도한다.</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>Hand Dominance Increase
 Hands Take Control</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>flip_release
 casting
 hand_dominance_increase</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="12" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>The Head Remains On The Trail Side.</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>머리가 트레일측에 남는다.</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr"/>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="D71" s="4" t="inlineStr"/>
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>head_hanging_back</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="F71" s="4" t="inlineStr">
         <is>
           <t>P6 신규. Head 수평축(위치) 링크.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="12" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>The Head Rises As The Body Stands Up.</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>몸이 일어나면서 머리가 상승한다.</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr"/>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr"/>
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>head_elevation
 spine_extension_excessive</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="F72" s="4" t="inlineStr">
         <is>
           <t>P6 신규. Early Extension/Spine → Head Elevation 공통 링크.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="12" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>The Lead Arm Cannot Extend Through Impact.</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>리드암이 임팩트 구간에서 충분히 뻗지 못한다.</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Chicken Wing Mechanism</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>hands_too_close_to_body
+steep_shaft
+trail_elbow_behind_body</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>P6 신규. Chicken Wing 링크.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>The Lead Arm Separates From The Thorax.</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>리드암이 몸통과 분리된다.</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D74" s="4" t="inlineStr">
         <is>
           <t>Chicken Wing
 Lead Arm Flies Off Chest</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr"/>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr"/>
+      <c r="F74" s="4" t="inlineStr">
         <is>
           <t>시트 M007. Chicken Wing 전조. P7 연계용 예약.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="12" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>The Swing Axis Shifts Upward.</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>회전축이 위로 이동한다.</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr"/>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="D75" s="4" t="inlineStr"/>
+      <c r="E75" s="4" t="inlineStr">
         <is>
           <t>head_elevation</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="F75" s="4" t="inlineStr">
         <is>
           <t>P6 신규.</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="12" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B70" s="4" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>The Torso Extends Backward To Recover Balance.</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>균형 회복을 위해 상체가 뒤로 신전한다.</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr"/>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="D76" s="4" t="inlineStr"/>
+      <c r="E76" s="4" t="inlineStr">
         <is>
           <t>spine_extension_excessive
 head_elevation</t>
         </is>
       </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="F76" s="4" t="inlineStr">
         <is>
           <t>P6 신규. Head/Spine 자세 보상 도메인.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="12" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>The Torso Flexes Excessively And The Head Drops.</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C77" s="4" t="inlineStr">
         <is>
           <t>상체가 과도하게 굴곡되며 머리가 낮아진다.</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr"/>
-      <c r="E71" s="4" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr"/>
+      <c r="E77" s="4" t="inlineStr">
         <is>
           <t>head_drop</t>
         </is>
       </c>
-      <c r="F71" s="4" t="inlineStr">
+      <c r="F77" s="4" t="inlineStr">
         <is>
           <t>P6 신규. Head Drop Flexion type.</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="12" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B72" s="4" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>The Trail Arm Extends Early To Deliver The Club.</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>클럽 전달을 위해 트레일 팔이 일찍 펴진다.</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>Right Arm Straightens Early
 Early Trail Arm Extension</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="E78" s="4" t="inlineStr">
         <is>
           <t>casting</t>
         </is>
       </c>
-      <c r="F72" s="4" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="12" t="inlineStr">
+      <c r="F78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
         <is>
           <t>CMP</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>The Trail Elbow Collapses Toward The Body.</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>트레일 팔꿈치가 몸통 쪽으로 급격하게 붙는다.</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t>Trail Elbow Pinch
 Right Elbow Jams In</t>
         </is>
       </c>
-      <c r="E73" s="4" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t>arm_stuck</t>
         </is>
       </c>
-      <c r="F73" s="4" t="inlineStr">
+      <c r="F79" s="4" t="inlineStr">
         <is>
           <t>시트 M006.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F73"/>
+  <autoFilter ref="A1:F79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6619,7 +8265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7746,8 +9392,288 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>Chicken Wing Pattern</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>치킨윙 패턴</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>임팩트 구간에서 리드암이 충분히 신전되지 못하고 굽혀지는 패턴. 공간·전달 실패의 보상.</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Pattern
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Inside Delivery</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>인사이드 딜리버리</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>클럽이 정상보다 안쪽 경로로 접근하는 전달 패턴.</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Path, Inside
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Over The Top</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>오버 더 탑</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>클럽이 전달 평면 위/바깥으로 넘어가며 접근하는 패턴 (Outside Delivery 계열).</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Path, Outside
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>Trail Elbow Flying</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>플라잉 엘보</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>트레일 팔꿈치가 몸통에서 과도하게 벌어지는(뜨는) 현상.</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>Trail Elbow</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Position, Wide
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>Shaft Lay Down</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>샤프트 눕힘</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>샤프트가 과도하게 눕는(수평화되는) 현상. Shallow Shaft의 극단.</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>Shaft</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Orientation, Lay Down
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>Handle Deep</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>핸들 깊음</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>그립 핸들이 정상보다 깊은(몸 뒤쪽) 위치에 있는 현상.</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>Shaft</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Position, Depth, Deep
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>High Angle Of Attack</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>높은 어택앵글</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>클럽헤드가 정상보다 수직에 가까운 경로로 임팩트에 접근하는 결과.</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Impact
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>Push Tendency</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>푸시 경향</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>스윙 방향 대비 클럽페이스 전달이 늦어 볼이 우측으로 밀리는 경향.</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Ball Flight
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>Impact Consistency Decrease</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>임팩트 일관성 감소</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>클럽 전달이 팔 타이밍에 의존하며 임팩트 일관성이 낮아지는 결과.</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Impact
+[status] pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>Lead Arm Separation Increase</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>리드암-흉곽 분리 증가</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>리드암과 흉곽의 연결이 약해져 분리가 증가하는 현상.</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Relationship
+[status] pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E40"/>
+  <autoFilter ref="A1:E50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8729,14 +10655,14 @@
           <t>Low Hands (손 낮음)</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8754,14 +10680,14 @@
           <t>Deep Hands (손 깊음)</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8779,14 +10705,14 @@
           <t>Forward Hands (손 전방)</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8804,14 +10730,14 @@
           <t>Hands Too Far From Body (손이 몸에서 멀어짐)</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8829,14 +10755,14 @@
           <t>Hands Too Close To Body (손이 몸에 가까움)</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8854,14 +10780,14 @@
           <t>Late Arm (팔 하강 지연)</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8879,14 +10805,14 @@
           <t>Trail Elbow Behind Body (트레일 팔꿈치 뒤처짐)</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8904,14 +10830,14 @@
           <t>Steep Shaft (가파른 샤프트)</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8929,14 +10855,14 @@
           <t>Shallow Shaft (눕는 샤프트)</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
@@ -8954,19 +10880,19 @@
           <t>Casting (캐스팅)</t>
         </is>
       </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>todo</t>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>원본 P6 기준 표준화 예정</t>
+          <t>6섹션 표준화 완료</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="C31" s="21" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>작업 순서(권장): Pelvis → Thorax → Pressure → Hands → Arm → Shaft → Club</t>
         </is>
@@ -8975,7 +10901,7 @@
     <row r="32">
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Phase 2-1: 모든 P6 Feature 6섹션 표준화 (진행 중)</t>
+          <t>Phase 2-1: 모든 P6 Feature 6섹션 표준화 (28/28 완료 ✅)</t>
         </is>
       </c>
     </row>

</xml_diff>